<commit_message>
add score calculator for response to evaluator prompt
</commit_message>
<xml_diff>
--- a/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
+++ b/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>alternate_abbreviation_status</t>
+          <t>alternate_abbreviation_status_w_no_context</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -518,7 +518,7 @@
     Primary gene symbol: TUB
     Official HGNC gene name: TUB bipartite transcription factor
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -538,9 +538,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "rd5",
+    "primary_gene_symbol": "TUB",
+    "name": "TUB bipartite transcription factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -600,7 +600,7 @@
     Primary gene symbol: BAG6
     Official HGNC gene name: BAG cochaperone 6
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -620,9 +620,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "SCYTHE",
+    "primary_gene_symbol": "BAG6",
+    "name": "BAG cochaperone 6",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -682,7 +682,7 @@
     Primary gene symbol: A4GNT
     Official HGNC gene name: alpha-1,4-N-acetylglucosaminyltransferase
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -702,9 +702,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ALPHA4GNT",
+    "primary_gene_symbol": "A4GNT",
+    "name": "alpha-1,4-N-acetylglucosaminyltransferase",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -764,7 +764,7 @@
     Primary gene symbol: A4GALT
     Official HGNC gene name: alpha 1,4-galactosyltransferase (P1PK blood group)
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -784,9 +784,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "A4GALT1",
+    "primary_gene_symbol": "A4GALT",
+    "name": "alpha 1,4-galactosyltransferase (P1PK blood group)",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -846,7 +846,7 @@
     Primary gene symbol: A4GALT
     Official HGNC gene name: alpha 1,4-galactosyltransferase (P1PK blood group)
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -866,9 +866,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "GB3S",
+    "primary_gene_symbol": "A4GALT",
+    "name": "alpha 1,4-galactosyltransferase (P1PK blood group)",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -928,7 +928,7 @@
     Primary gene symbol: AANAT
     Official HGNC gene name: aralkylamine N-acetyltransferase
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -948,9 +948,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "SNAT",
+    "primary_gene_symbol": "AANAT",
+    "name": "aralkylamine N-acetyltransferase",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1010,7 +1010,7 @@
     Primary gene symbol: MED23
     Official HGNC gene name: mediator complex subunit 23
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1030,9 +1030,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "SUR-2",
+    "primary_gene_symbol": "MED23",
+    "name": "mediator complex subunit 23",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1092,7 +1092,7 @@
     Primary gene symbol: A1CF
     Official HGNC gene name: APOBEC1 complementation factor
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1112,9 +1112,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ACF",
+    "primary_gene_symbol": "A1CF",
+    "name": "APOBEC1 complementation factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1174,7 +1174,7 @@
     Primary gene symbol: A1CF
     Official HGNC gene name: APOBEC1 complementation factor
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1194,9 +1194,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ACF64",
+    "primary_gene_symbol": "A1CF",
+    "name": "APOBEC1 complementation factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1256,7 +1256,7 @@
     Primary gene symbol: A1CF
     Official HGNC gene name: APOBEC1 complementation factor
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1276,9 +1276,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ACF65",
+    "primary_gene_symbol": "A1CF",
+    "name": "APOBEC1 complementation factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="G12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1338,7 +1338,7 @@
     Primary gene symbol: A1CF
     Official HGNC gene name: APOBEC1 complementation factor
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1358,9 +1358,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ASP",
+    "primary_gene_symbol": "A1CF",
+    "name": "APOBEC1 complementation factor",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1420,7 +1420,7 @@
     Primary gene symbol: A3GALT2
     Official HGNC gene name: alpha 1,3-galactosyltransferase 2
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1440,9 +1440,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "IGB3S",
+    "primary_gene_symbol": "A3GALT2",
+    "name": "alpha 1,3-galactosyltransferase 2",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="G14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1502,7 +1502,7 @@
     Primary gene symbol: SNORA36B
     Official HGNC gene name: small nucleolar RNA, H/ACA box 36B
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1522,9 +1522,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ACA36b",
+    "primary_gene_symbol": "SNORA36B",
+    "name": "small nucleolar RNA, H/ACA box 36B",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
       <c r="G15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1584,7 +1584,7 @@
     Primary gene symbol: FOLR3
     Official HGNC gene name: folate receptor gamma
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1604,9 +1604,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "FRgamma",
+    "primary_gene_symbol": "FOLR3",
+    "name": "folate receptor gamma",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1666,7 +1666,7 @@
     Primary gene symbol: A1BG
     Official HGNC gene name: alpha-1-B glycoprotein
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1686,9 +1686,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "A1B",
+    "primary_gene_symbol": "A1BG",
+    "name": "alpha-1-B glycoprotein",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1748,7 +1748,7 @@
     Primary gene symbol: A1BG
     Official HGNC gene name: alpha-1-B glycoprotein
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1768,9 +1768,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ABG",
+    "primary_gene_symbol": "A1BG",
+    "name": "alpha-1-B glycoprotein",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1830,7 +1830,7 @@
     Primary gene symbol: A1BG
     Official HGNC gene name: alpha-1-B glycoprotein
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1850,9 +1850,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "GAB",
+    "primary_gene_symbol": "A1BG",
+    "name": "alpha-1-B glycoprotein",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1912,7 +1912,7 @@
     Primary gene symbol: KRT7
     Official HGNC gene name: keratin 7
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -1932,9 +1932,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "SCL",
+    "primary_gene_symbol": "KRT7",
+    "name": "keratin 7",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -1994,7 +1994,7 @@
     Primary gene symbol: LMAN1
     Official HGNC gene name: lectin, mannose binding 1
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -2014,9 +2014,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "GP58",
+    "primary_gene_symbol": "LMAN1",
+    "name": "lectin, mannose binding 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2076,7 +2076,7 @@
     Primary gene symbol: CIITA
     Official HGNC gene name: class II major histocompatibility complex transactivator
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -2096,9 +2096,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "NLRA",
+    "primary_gene_symbol": "CIITA",
+    "name": "class II major histocompatibility complex transactivator",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2158,7 +2158,7 @@
     Primary gene symbol: ABCG2
     Official HGNC gene name: ATP binding cassette subfamily G member 2 (JR blood group)
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -2178,9 +2178,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "CD338",
+    "primary_gene_symbol": "ABCG2",
+    "name": "ATP binding cassette subfamily G member 2 (JR blood group)",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2240,7 +2240,7 @@
     Primary gene symbol: AOC1
     Official HGNC gene name: amine oxidase copper containing 1
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -2260,9 +2260,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "ABP1",
+    "primary_gene_symbol": "AOC1",
+    "name": "amine oxidase copper containing 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>
@@ -2322,7 +2322,7 @@
     Primary gene symbol: RBMXP1
     Official HGNC gene name: RBMX pseudogene 1
     Task:
-    Determine whether it is possible that the alias symbol is an abbreviation variant of the official HGNC gene name. 
+    Determine whether the alias symbol is an abbreviation variant of the official HGNC gene name. 
     Classify the alias symbol as an Alternate Abbreviation only if the letters are reasonably able to be expanded to the official
     HGNC gene name, or to a phrase that is nearly identical in wording and meaning.
     Examples:
@@ -2342,9 +2342,9 @@
     Output only one JSON object. No markdown.
     {
     "pmid": "",
-    "alias_symbol": "",
-    "primary_gene_symbol": "",
-    "name": "",
+    "alias_symbol": "HNRNP-G",
+    "primary_gene_symbol": "RBMXP1",
+    "name": "RBMX pseudogene 1",
     "alternate_abbreviation": "TRUE or FALSE"
     }</t>
         </is>

</xml_diff>

<commit_message>
repeated a run with the same prompt for robustness testing. first run was 86%P and 96%R. this second run was 84%P and 93%R
</commit_message>
<xml_diff>
--- a/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
+++ b/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
@@ -825,7 +825,7 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>{
-"reason": "U51 is not an alternate abbreviation of 'small nucleolar RNA, C/D box 51' as it does not represent the same description using different letters.",
+"reason": "U51 is not an alternate abbreviation of the official gene name as it does not represent the same description using different letters.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -911,7 +911,7 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>{
-"reason": "RPL36A is not an alternate abbreviation of 'ribosomal protein L36a like' because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
+"reason": "RPL36A is not an alternate abbreviation because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1418,7 +1418,7 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>{
-"reason": "ARALAR1 is not derived from the official gene name or primary symbol, but appears to be a distinct alias representing a different aspect of the gene.",
+"reason": "ARALAR1 is not derived from the official gene name 'solute carrier family 25 member 12' or the primary symbol SLC25A12, but appears to be a different description or name for the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -2008,7 +2008,7 @@
       <c r="L19" t="inlineStr">
         <is>
           <t>{
-"reason": "TGFR-1 is an alternate abbreviation of the official gene name as it represents 'transforming growth factor receptor 1' with a different letter combination.",
+"reason": "TGFR-1 is an alternate abbreviation of the official gene name as it represents 'transforming growth factor receptor 1' with a different letter arrangement.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2343,7 +2343,7 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>{
-"reason": "TCRBV11S3 is an alternate abbreviation of T cell receptor beta variable 11-3, as it uses different letters to represent the same gene name components.",
+"reason": "TCRBV11S3 is an alternate abbreviation of the official gene name as it represents 'T cell receptor beta variable 11-3' using different letters and formatting.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2927,7 +2927,7 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>{
-"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene name but with one letter omitted.",
+"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene but with the 'H' omitted.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -3597,7 +3597,7 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>{
-"reason": "RI58 does not appear to be derived from the letters in the official gene name or primary symbol IFIT5.",
+"reason": "RI58 does not appear to be derived from the official gene name or primary symbol IFIT5, and likely represents a different description or naming convention for the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4522,7 +4522,7 @@
       <c r="L49" t="inlineStr">
         <is>
           <t>{
-"reason": "CLEC4N is not an alternate abbreviation of the official gene name 'C-type lectin domain containing 6A' as it contains a different number (4) than the primary symbol (6).",
+"reason": "CLEC4N is not an alternate abbreviation of the official gene name as it contains a different number (4) than the primary gene symbol (6).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4608,7 +4608,7 @@
       <c r="L50" t="inlineStr">
         <is>
           <t>{
-"reason": "DECTIN1 is not an abbreviation variant of the official gene name 'C-type lectin domain containing 7A' as it represents a different description of the gene.",
+"reason": "DECTIN1 is not derived from the official gene name 'C-type lectin domain containing 7A' or the primary symbol CLEC7A, but rather represents a different description of the gene's function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4694,7 +4694,7 @@
       <c r="L51" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol OR10AC1P is not an alternate abbreviation because it includes a 'P' at the end, which is not present in the official gene name and likely indicates a pseudogene variant.",
+"reason": "The alias symbol OR10AC1P is not an alternate abbreviation because it includes an additional 'P' at the end, which is not present in the official gene name or primary symbol and likely indicates a pseudogene variant.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4780,7 +4780,7 @@
       <c r="L52" t="inlineStr">
         <is>
           <t>{
-"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, as it uses 'H' instead of 'L' but still represents the same gene concept.",
+"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, where 'H' likely stands for 'homolog' or 'human', which is not present in the official gene name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -5619,7 +5619,7 @@
       <c r="L62" t="inlineStr">
         <is>
           <t>{
-"reason": "UNCL is not an alternate abbreviation of the official gene name as it does not represent the same name with different letters and appears to be a shortened version of UNC50, which could potentially represent a family name.",
+"reason": "UNCL is not an alternate abbreviation of the official gene name as it lacks the number '50' which is present in the primary gene symbol UNC50.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -5705,7 +5705,7 @@
       <c r="L63" t="inlineStr">
         <is>
           <t>{
-"reason": "ACECS2L is not an alternate abbreviation of 'acyl-CoA synthetase short chain family member 1' as it contains characters (E, C, 2, L) not present in the official gene name.",
+"reason": "ACECS2L is not an alternate abbreviation of the official gene name as it contains additional characters (E and 2) not present in the official name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6292,7 +6292,7 @@
       <c r="L70" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '4E-T' is an abbreviated form of 'eIF4E transporter' which is not present in the official gene name, so it is not an alternate abbreviation of the official name.",
+"reason": "The alias symbol '4E-T' is not derived from the letters in the official gene name, but rather appears to be a different description or representation of the gene's function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6461,7 +6461,7 @@
       <c r="L72" t="inlineStr">
         <is>
           <t>{
-"reason": "PDZD5A is not an alternate abbreviation of the official gene name as it represents a different description of the gene, focusing on the PDZ domain rather than the FERM and PDZ domains mentioned in the full name.",
+"reason": "PDZD5A is not an alternate abbreviation of the official gene name as it only represents a part of the gene's function (PDZ domain) and does not include the FERM domain or indicate it's a pseudogene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6630,7 +6630,7 @@
       <c r="L74" t="inlineStr">
         <is>
           <t>{
-"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' or CNMD, as it appears to be derived from a different description or previous name of the gene.",
+"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' as it contains letters not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6971,7 +6971,7 @@
       <c r="L78" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'hPot1' is an alternate abbreviation of the official gene name, as it includes the 'h' prefix (likely for 'human') and capitalizes the second letter, but otherwise represents the same gene.",
+"reason": "The alias symbol 'hPot1' is an alternate abbreviation of the official gene name as it includes the 'h' prefix for human and capitalizes only the first letter of 'Pot', while maintaining the same meaning.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -7810,7 +7810,7 @@
       <c r="L88" t="inlineStr">
         <is>
           <t>{
-"reason": "ALPHA4GNT is an alternate abbreviation of the official gene name as it spells out 'ALPHA' instead of using 'A' in the primary symbol, but represents the same gene.",
+"reason": "ALPHA4GNT is an alternate abbreviation of the official gene name as it represents the same enzyme using 'ALPHA' instead of 'A' for 'alpha'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -8145,7 +8145,7 @@
       <c r="L92" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol A4GALT1 is not an alternate abbreviation because it includes an additional '1' at the end, which is not present in the official gene name or primary symbol.",
+"reason": "A4GALT1 is not an alternate abbreviation because it includes an additional '1' that is not present in the official gene name or primary gene symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -8812,7 +8812,7 @@
       <c r="L100" t="inlineStr">
         <is>
           <t>{
-"reason": "KRTAP8P2 is not an alternate abbreviation because it represents a different gene (KRTAP8-2) than the official gene name (KRTAP8-3P), as indicated by the different number after the name.",
+"reason": "KRTAP8P2 is not an alternate abbreviation because it represents a different gene (KRTAP8-2) than the official gene name (KRTAP8-3).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -9568,8 +9568,8 @@
       <c r="L109" t="inlineStr">
         <is>
           <t>{
-"reason": "HMGB1L14 is an alternate abbreviation of the official gene name because it represents the same gene with a slight variation in the pseudogene designation (L instead of P).",
-"alternate_abbreviation": "TRUE"
+"reason": "The alias symbol HMGB1L14 is not an alternate abbreviation because it uses 'L' instead of 'P' to represent 'pseudogene', which is not consistent with the official gene name.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -10733,7 +10733,7 @@
       <c r="L123" t="inlineStr">
         <is>
           <t>{
-"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and appears to represent a different aspect of the gene.",
+"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and appears to represent a different concept or description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -11483,7 +11483,7 @@
       <c r="L132" t="inlineStr">
         <is>
           <t>{
-"reason": "CPU is not an alternate abbreviation of carboxypeptidase B2 as it does not represent the same gene name using different letters.",
+"reason": "CPU is not an alternate abbreviation of carboxypeptidase B2 as it does not use letters from the official gene name in the same order.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12406,7 +12406,7 @@
       <c r="L143" t="inlineStr">
         <is>
           <t>{
-"reason": "ACF is an alternate abbreviation of the official gene name APOBEC1 complementation factor, using the first letter of each word.",
+"reason": "ACF is an alternate abbreviation of the official gene name 'APOBEC1 complementation factor' as it uses the first letter of each word.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -12830,7 +12830,7 @@
       <c r="L148" t="inlineStr">
         <is>
           <t>{
-"reason": "SYN is an alternate abbreviation of synemin as it uses the first three letters of the official gene name.",
+"reason": "SYN is an alternate abbreviation of synemin as it represents a shortened version of the official gene name without adding any new characters.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -15501,7 +15501,7 @@
       <c r="L180" t="inlineStr">
         <is>
           <t>{
-"reason": "CSTF3-AS1 is not an alternate abbreviation because 'AS1' stands for 'antisense RNA 1', which is a different description from the official gene name 'CSTF3 divergent transcript'.",
+"reason": "The alias symbol CSTF3-AS1 is not an alternate abbreviation of the official gene name 'CSTF3 divergent transcript' as it represents a different description (antisense RNA) rather than an abbreviation variant.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -18012,7 +18012,7 @@
       <c r="L210" t="inlineStr">
         <is>
           <t>{
-"reason": "WFIKKN is an alternate abbreviation of the official gene name as it represents the same gene without the number '1' at the end.",
+"reason": "WFIKKN is an alternate abbreviation of the official gene name as it represents the same gene but without the number '1' at the end.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18181,7 +18181,7 @@
       <c r="L212" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN139 is an alternate abbreviation of microRNA 139, as it uses 'MIRN' instead of 'MIR' but still represents the same gene.",
+"reason": "MIRN139 is an alternate abbreviation of microRNA 139, as it uses 'MIRN' instead of 'MIR' to represent 'microRNA'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18353,7 +18353,7 @@
       <c r="L214" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'A' at the end.",
+"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'a' at the end.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18780,7 +18780,7 @@
       <c r="L219" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'mir-491' is an alternate abbreviation of the official gene name 'microRNA 491' as it represents the same gene with a slight variation in capitalization and the use of a hyphen.",
+"reason": "The alias symbol 'mir-491' is a lowercase version of the primary gene symbol 'MIR491' and represents the same microRNA gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18949,7 +18949,7 @@
       <c r="L221" t="inlineStr">
         <is>
           <t>{
-"reason": "RanBP2L2 is not an alternate abbreviation of the official gene name because it represents a different description of the gene (RAN binding protein 2-like 2) rather than an abbreviation of 'RANBP2 like and GRIP domain containing 6'.",
+"reason": "RanBP2L2 is not an alternate abbreviation of the official gene name because it represents a different description of the gene (RANBP2 like) without including the GRIP domain or the number 6.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -19290,7 +19290,7 @@
       <c r="L225" t="inlineStr">
         <is>
           <t>{
-"reason": "ACA31 is an alternate abbreviation of the official gene name 'small nucleolar RNA, H/ACA box 31' as it represents the 'ACA box' portion of the name.",
+"reason": "ACA31 is an alternate abbreviation of the official gene name as it represents the 'H/ACA box' part of 'small nucleolar RNA, H/ACA box 31'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -19459,7 +19459,7 @@
       <c r="L227" t="inlineStr">
         <is>
           <t>{
-"reason": "ACA36b is an alternate abbreviation of the official gene name as it represents 'H/ACA box 36B' from the full name 'small nucleolar RNA, H/ACA box 36B'.",
+"reason": "ACA36b is an alternate abbreviation of the official gene name as it represents 'H/ACA box 36B' from the full name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -19963,7 +19963,7 @@
       <c r="L233" t="inlineStr">
         <is>
           <t>{
-"reason": "ELA1 is an alternate abbreviation of the official gene name 'chymotrypsin like elastase 1' as it uses the first letter of 'elastase' and the number '1' from the full name.",
+"reason": "ELA1 is an alternate abbreviation of the official gene name 'chymotrypsin like elastase 1' as it uses the first letter of 'elastase' and '1' from the name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20132,7 +20132,7 @@
       <c r="L235" t="inlineStr">
         <is>
           <t>{
-"reason": "CT45-4 is not an alternate abbreviation because it represents a different member of the CT45 family (CT45-4) compared to the official gene (CT45A5).",
+"reason": "CT45-4 is not an alternate abbreviation because it represents a different member of the CT45 family (CT45-4) rather than the specific gene CT45A5.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -20553,7 +20553,7 @@
       <c r="L240" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'tRNA-Asp-GTC-2-5' is an exact match to the official gene name 'tRNA-Asp (anticodon GTC) 2-5' with only minor formatting differences.",
+"reason": "The alias symbol 'tRNA-Asp-GTC-2-5' is an exact match to the official HGNC gene name 'tRNA-Asp (anticodon GTC) 2-5' with only minor formatting differences.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -21069,7 +21069,7 @@
       <c r="L246" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN1185-1 is an alternate abbreviation of microRNA 1185-1 because it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while maintaining the same numerical identifier.",
+"reason": "MIRN1185-1 is an alternate abbreviation of microRNA 1185-1 because it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while maintaining the same numeric identifier.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -21155,8 +21155,8 @@
       <c r="L247" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol HSA-MIR-548H-1 is an alternate abbreviation of the official gene name 'microRNA 548h-1' with added hyphens and 'HSA' prefix.",
-"alternate_abbreviation": "TRUE"
+"reason": "The alias symbol HSA-MIR-548H-1 is not an alternate abbreviation because it contains additional characters (HSA- and -) that are not present in the official gene name or primary symbol.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -21241,7 +21241,7 @@
       <c r="L248" t="inlineStr">
         <is>
           <t>{
-"reason": "PAR1 is not derived from the official gene name 'coagulation factor II thrombin receptor' or the primary symbol 'F2R', but rather represents a different description of the gene (Protease-Activated Receptor 1).",
+"reason": "PAR1 is not derived from the official gene name 'coagulation factor II thrombin receptor' or the primary symbol F2R, but rather stands for 'protease-activated receptor 1', which is a different description of the gene's function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21410,7 +21410,7 @@
       <c r="L250" t="inlineStr">
         <is>
           <t>{
-"reason": "FAT is not an alternate abbreviation because it is a shortened version of the primary gene symbol FAT1, likely representing a family name rather than a specific gene.",
+"reason": "FAT is not an alternate abbreviation because it is a shortened version of the primary gene symbol FAT1, which likely represents a gene family name rather than an abbreviation variant of the specific gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21748,7 +21748,7 @@
       <c r="L254" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, making it not an alternate abbreviation.",
+"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L26 pseudogene 30'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22086,7 +22086,7 @@
       <c r="L258" t="inlineStr">
         <is>
           <t>{
-"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because the number 9 in the alias symbol does not correspond to the 1B in the official gene name.",
+"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because it represents a different member of the FKBP family (FKBP9 vs FKBP1B).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22341,7 +22341,7 @@
       <c r="L261" t="inlineStr">
         <is>
           <t>{
-"reason": "FRgamma is an alternate abbreviation of 'folate receptor gamma' using the first letters of each word.",
+"reason": "FRgamma is an alternate abbreviation as it represents 'folate receptor gamma' using different letters (FR) than the primary symbol (FOLR3).",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -22845,7 +22845,7 @@
       <c r="L267" t="inlineStr">
         <is>
           <t>{
-"reason": "TH2-LCR is an alternate abbreviation of the official gene name as it represents the same concept with a hyphen instead of the full 'R' for 'region' at the end.",
+"reason": "TH2-LCR is an alternate abbreviation of the official gene name as it represents the same concept with a hyphen instead of the word 'associated' and 'RNA'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -23850,7 +23850,7 @@
       <c r="L279" t="inlineStr">
         <is>
           <t>{
-"reason": "RN5S434 is an alternate abbreviation of RNA5SP434, as it represents the same gene with a shortened form of the primary symbol.",
+"reason": "RN5S434 is an alternate abbreviation of RNA, 5S ribosomal pseudogene 434 as it uses different letters to represent the same gene name components.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -24437,7 +24437,7 @@
       <c r="L286" t="inlineStr">
         <is>
           <t>{
-"reason": "GSHPx-3 is an alternate abbreviation of glutathione peroxidase 3, as it includes 'GSH' for glutathione, 'Px' for peroxidase, and '3' for the specific isoform number.",
+"reason": "GSHPx-3 is an alternate abbreviation of glutathione peroxidase 3, as it represents the same enzyme with a different abbreviation style.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -24941,7 +24941,7 @@
       <c r="L292" t="inlineStr">
         <is>
           <t>{
-"reason": "SCHAD is not derived from the letters in the official gene name 'hydroxysteroid 17-beta dehydrogenase 10' or the primary symbol 'HSD17B10', suggesting it represents a different description of the gene.",
+"reason": "SCHAD is not derived from the letters in the official gene name 'hydroxysteroid 17-beta dehydrogenase 10' or the primary symbol 'HSD17B10'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25362,7 +25362,7 @@
       <c r="L297" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'onco-lncRNA-32' is not an alternate abbreviation of the official gene name as it includes additional descriptive elements ('onco' and '32') not present in the official name or primary symbol.",
+"reason": "The alias symbol 'onco-lncRNA-32' is not an abbreviation variant of the official gene name as it includes additional information ('onco') and a different number ('32') not present in the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25448,7 +25448,7 @@
       <c r="L298" t="inlineStr">
         <is>
           <t>{
-"reason": "A1B is a shortened version of the primary gene symbol A1BG, representing the same gene without changing the meaning.",
+"reason": "A1B is a shortened version of the primary gene symbol A1BG, representing the same gene without altering the meaning.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -26622,7 +26622,7 @@
       <c r="L312" t="inlineStr">
         <is>
           <t>{
-"reason": "V1-17 is not an alternate abbreviation of 'immunoglobulin lambda variable 1-47' as it represents a different numbered variant of the gene family.",
+"reason": "V1-17 is not an alternate abbreviation of IGLV1-47 or immunoglobulin lambda variable 1-47 because it represents a different numbered variant of the gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -26874,7 +26874,7 @@
       <c r="L315" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' as it includes a hyphen between IL and 12A but represents the same gene.",
+"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' with a hyphen added between IL and 12A.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -27043,7 +27043,7 @@
       <c r="L317" t="inlineStr">
         <is>
           <t>{
-"reason": "ITGB1BP is not an alternate abbreviation because it lacks the number '2' present in both the primary gene symbol and official gene name, potentially representing a different gene or family member.",
+"reason": "ITGB1BP is not an alternate abbreviation because it is a shortened version of the primary gene symbol ITGB1BP2, likely representing a family name rather than the specific gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -27298,7 +27298,7 @@
       <c r="L320" t="inlineStr">
         <is>
           <t>{
-"reason": "EKLF is an alternate abbreviation for 'Erythroid Kruppel-like Factor', which is a previous name for KLF1, while KLF1 is the primary gene symbol.",
+"reason": "EKLF is an alternate abbreviation for 'Erythroid Kruppel-like Factor', which is a previous name for KLF1, while KLF1 is the current primary gene symbol.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -27384,8 +27384,8 @@
       <c r="L321" t="inlineStr">
         <is>
           <t>{
-"reason": "IPOA7 is an alternate abbreviation for 'importin alpha 7', which is a different description of the gene's function compared to the official name 'karyopherin subunit alpha 6'.",
-"alternate_abbreviation": "FALSE"
+"reason": "IPOA7 is an alternate abbreviation for 'importin alpha 7', which is a previous name for karyopherin subunit alpha 6.",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -27885,7 +27885,7 @@
       <c r="L327" t="inlineStr">
         <is>
           <t>{
-"reason": "SAMS1 is not an alternate abbreviation of 'methionine adenosyltransferase 1A' as it represents a different description of the gene (S-adenosylmethionine synthetase 1) rather than a variant abbreviation of the official name.",
+"reason": "SAMS1 is not derived from the letters in the official gene name 'methionine adenosyltransferase 1A' or the primary symbol MAT1A, but appears to represent a different description of the gene's function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -28893,7 +28893,7 @@
       <c r="L339" t="inlineStr">
         <is>
           <t>{
-"reason": "NFIB3 is not an alternate abbreviation because it contains a number (3) that is not present in the official gene name 'nuclear factor I B'.",
+"reason": "NFIB3 is not an alternate abbreviation because it includes a number (3) that is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29234,7 +29234,7 @@
       <c r="L343" t="inlineStr">
         <is>
           <t>{
-"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains characters (L and 211) not present in 'olfactory receptor family 1 subfamily C member 1'.",
+"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains an 'L' which is not present in the official name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30322,7 +30322,7 @@
       <c r="L356" t="inlineStr">
         <is>
           <t>{
-"reason": "Pr1/Pr2 is not an alternate abbreviation of the official gene name as it represents different gene numbers (1 and 2) compared to the primary gene symbol PRH1.",
+"reason": "Pr1/Pr2 is not an alternate abbreviation of 'proline rich protein HaeIII subfamily 1' as it represents different subfamily members (1 and 2) rather than an abbreviation of the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -31078,8 +31078,8 @@
       <c r="L365" t="inlineStr">
         <is>
           <t>{
-"reason": "RECC1 is not an alternate abbreviation of 'replication factor C subunit 1' as it contains a 'C' not present in the official gene name.",
-"alternate_abbreviation": "FALSE"
+"reason": "RECC1 is an alternate abbreviation for 'replication factor C subunit 1' using different letters to represent the same concept as RFC1.",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>

</xml_diff>

<commit_message>
third run for rubustinity testing, 86%P and 93%R
</commit_message>
<xml_diff>
--- a/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
+++ b/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
@@ -570,7 +570,7 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>{
-"reason": "RHPII is not an alternate abbreviation as it contains additional characters (PII) not present in the official gene name or primary symbol.",
+"reason": "RHPII is not an alternate abbreviation of 'Rh blood group D antigen' as it contains additional characters (PII) not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -656,7 +656,7 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RN7SL427P is not an alternate abbreviation of the official gene name because it contains the number 427, which is not present in the official gene name or primary symbol.",
+"reason": "The alias symbol RN7SL427P is not an alternate abbreviation of the official gene name because it contains the number '427' which is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -825,7 +825,7 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>{
-"reason": "U51 is not an alternate abbreviation of the official gene name as it does not represent the same description using different letters.",
+"reason": "U51 is not an alternate abbreviation of the official gene name or primary symbol, as it represents a different description or classification of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -911,7 +911,7 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>{
-"reason": "RPL36A is not an alternate abbreviation because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
+"reason": "RPL36A is not an alternate abbreviation of 'ribosomal protein L36a like' because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1163,7 +1163,7 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>{
-"reason": "MCT3 is not derived from the letters in the official gene name 'solute carrier family 16 member 3' and appears to be a different description or naming convention for the gene.",
+"reason": "MCT3 is an alternate abbreviation for 'monocarboxylate transporter 3', which is a different description of the gene and not directly related to the official name 'solute carrier family 16 member 3'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1332,7 +1332,7 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>{
-"reason": "HOCT1 is not derived from the letters in the official gene name 'solute carrier family 22 member 1' or the primary symbol SLC22A1, but appears to be a different description of the gene.",
+"reason": "HOCT1 is not derived from the letters in the official gene name 'solute carrier family 22 member 1' or the primary symbol SLC22A1, but rather appears to be a different description or acronym for the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1922,7 +1922,7 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>{
-"reason": "TRBF2 is an alternate abbreviation of 'telomeric repeat binding factor 2' using different letters to represent the same concept.",
+"reason": "TRBF2 is an alternate abbreviation of 'telomeric repeat binding factor 2' using different letters to represent the same concept as TERF2.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2343,7 +2343,7 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>{
-"reason": "TCRBV11S3 is an alternate abbreviation of the official gene name as it represents 'T cell receptor beta variable 11-3' using different letters and formatting.",
+"reason": "TCRBV11S3 is an alternate abbreviation of the official gene name as it represents the same T cell receptor beta variable gene with a slightly different numbering format.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2927,7 +2927,7 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>{
-"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene but with the 'H' omitted.",
+"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene but with the 'H' omitted from the primary symbol.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -3597,7 +3597,7 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>{
-"reason": "RI58 does not appear to be derived from the official gene name or primary symbol IFIT5, and likely represents a different description or naming convention for the gene.",
+"reason": "RI58 does not appear to be derived from the letters in the official gene name or primary symbol IFIT5.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -3683,7 +3683,7 @@
       <c r="L39" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'Ly-6D' is an alternate abbreviation of the primary gene symbol 'LY6D', differing only in the use of a hyphen and lowercase 'y'.",
+"reason": "The alias symbol 'Ly-6D' is an alternate abbreviation of the primary gene symbol 'LY6D' with only a minor difference in capitalization and hyphenation.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -3935,7 +3935,7 @@
       <c r="L42" t="inlineStr">
         <is>
           <t>{
-"reason": "CALS is not an alternate abbreviation of 'carbonic anhydrase 8 (inactive)' as it contains letters not present in the official gene name.",
+"reason": "CALS is not an alternate abbreviation of 'carbonic anhydrase 8' as it contains letters not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4522,7 +4522,7 @@
       <c r="L49" t="inlineStr">
         <is>
           <t>{
-"reason": "CLEC4N is not an alternate abbreviation of the official gene name as it contains a different number (4) than the primary gene symbol (6).",
+"reason": "CLEC4N is not an alternate abbreviation of the official gene name as it contains a different number (4) than the primary gene symbol (6), indicating it likely represents a different member of the CLEC family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4608,7 +4608,7 @@
       <c r="L50" t="inlineStr">
         <is>
           <t>{
-"reason": "DECTIN1 is not derived from the official gene name 'C-type lectin domain containing 7A' or the primary symbol CLEC7A, but rather represents a different description of the gene's function.",
+"reason": "DECTIN1 is not an alternate abbreviation of the official gene name 'C-type lectin domain containing 7A' as it represents a different description of the gene function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4780,7 +4780,7 @@
       <c r="L52" t="inlineStr">
         <is>
           <t>{
-"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, where 'H' likely stands for 'homolog' or 'human', which is not present in the official gene name.",
+"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, as it uses 'H' instead of 'L' but still represents the same gene concept.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -5705,7 +5705,7 @@
       <c r="L63" t="inlineStr">
         <is>
           <t>{
-"reason": "ACECS2L is not an alternate abbreviation of the official gene name as it contains additional characters (E and 2) not present in the official name or primary symbol.",
+"reason": "ACECS2L is not an alternate abbreviation of 'acyl-CoA synthetase short chain family member 1' as it contains additional characters (E, C, 2, L) not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6292,7 +6292,7 @@
       <c r="L70" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '4E-T' is not derived from the letters in the official gene name, but rather appears to be a different description or representation of the gene's function.",
+"reason": "The alias symbol '4E-T' is an abbreviated form of 'eIF4E transporter' which is not present in the official gene name, so it is not an alternate abbreviation of the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6630,7 +6630,7 @@
       <c r="L74" t="inlineStr">
         <is>
           <t>{
-"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' as it contains letters not present in the official gene name.",
+"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' or CNMD, as it appears to be derived from a different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6971,7 +6971,7 @@
       <c r="L78" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'hPot1' is an alternate abbreviation of the official gene name as it includes the 'h' prefix for human and capitalizes only the first letter of 'Pot', while maintaining the same meaning.",
+"reason": "The alias symbol 'hPot1' is an alternate abbreviation of the official gene name as it includes 'h' for human and capitalizes the first letter of 'Pot', while maintaining the same meaning.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -8898,7 +8898,7 @@
       <c r="L101" t="inlineStr">
         <is>
           <t>{
-"reason": "SNAT is an alternate abbreviation of the official gene name 'aralkylamine N-acetyltransferase' as it uses different letters to represent the same enzyme.",
+"reason": "SNAT is an alternate abbreviation of the official gene name 'aralkylamine N-acetyltransferase' as it uses different letters to represent the same concept.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -10733,7 +10733,7 @@
       <c r="L123" t="inlineStr">
         <is>
           <t>{
-"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and appears to represent a different concept or description of the gene.",
+"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and appears to represent a different aspect of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -11483,7 +11483,7 @@
       <c r="L132" t="inlineStr">
         <is>
           <t>{
-"reason": "CPU is not an alternate abbreviation of carboxypeptidase B2 as it does not use letters from the official gene name in the same order.",
+"reason": "CPU is not an alternate abbreviation of carboxypeptidase B2 as it does not represent the same gene name using different letters.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12011,9 +12011,7 @@
           <t>MED23</t>
         </is>
       </c>
-      <c r="E139" t="e">
-        <v>#NAME?</v>
-      </c>
+      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>mediator complex subunit 23</t>
@@ -12068,7 +12066,7 @@
       <c r="L139" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '#NAME?' does not appear to be an abbreviation variant of the official gene name 'mediator complex subunit 23' or the primary symbol 'MED23'.",
+"reason": "The alias symbol '#NAME?' is not a valid gene symbol and does not appear to be an abbreviation variant of the official gene name 'mediator complex subunit 23' or the primary symbol 'MED23'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12406,7 +12404,7 @@
       <c r="L143" t="inlineStr">
         <is>
           <t>{
-"reason": "ACF is an alternate abbreviation of the official gene name 'APOBEC1 complementation factor' as it uses the first letter of each word.",
+"reason": "ACF is an alternate abbreviation of the official gene name 'APOBEC1 complementation factor' as it uses the first letter of each word in the name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -12661,7 +12659,7 @@
       <c r="L146" t="inlineStr">
         <is>
           <t>{
-"reason": "CPX-IV is an alternate abbreviation of complexin 4, using 'CPX' for 'complexin' and 'IV' (Roman numeral 4) instead of '4'.",
+"reason": "CPX-IV is an alternate abbreviation of complexin 4, using 'CPX' instead of 'CPLX' and Roman numeral 'IV' instead of '4'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -12830,7 +12828,7 @@
       <c r="L148" t="inlineStr">
         <is>
           <t>{
-"reason": "SYN is an alternate abbreviation of synemin as it represents a shortened version of the official gene name without adding any new characters.",
+"reason": "SYN is an alternate abbreviation of synemin as it uses the first three letters of the official gene name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -15166,7 +15164,7 @@
       <c r="L176" t="inlineStr">
         <is>
           <t>{
-"reason": "EFO2p is not an alternate abbreviation of ESCO2 or the official gene name because it contains a 'p' which is not present in either the primary symbol or the official name.",
+"reason": "EFO2p is not an alternate abbreviation of ESCO2 or the official gene name, as it contains a 'p' which is not present in either the primary symbol or the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -15501,7 +15499,7 @@
       <c r="L180" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol CSTF3-AS1 is not an alternate abbreviation of the official gene name 'CSTF3 divergent transcript' as it represents a different description (antisense RNA) rather than an abbreviation variant.",
+"reason": "CSTF3-AS1 is not an alternate abbreviation because it represents a different description of the gene (antisense RNA) compared to the official gene name (divergent transcript).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -17677,7 +17675,7 @@
       <c r="L206" t="inlineStr">
         <is>
           <t>{
-"reason": "TESSP1 is not an alternate abbreviation of 'serine protease 41' as it appears to represent a different description or aspect of the gene.",
+"reason": "TESSP1 is not an alternate abbreviation of 'serine protease 41' as it appears to represent a different description or aspect of the gene rather than an abbreviation of the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -18012,8 +18010,8 @@
       <c r="L210" t="inlineStr">
         <is>
           <t>{
-"reason": "WFIKKN is an alternate abbreviation of the official gene name as it represents the same gene but without the number '1' at the end.",
-"alternate_abbreviation": "TRUE"
+"reason": "WFIKKN is not an alternate abbreviation because it is a shortened version of the primary gene symbol WFIKKN1, likely representing a family name rather than a specific gene.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -18353,7 +18351,7 @@
       <c r="L214" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'a' at the end.",
+"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'A' at the end.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18694,7 +18692,7 @@
       <c r="L218" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN410 is an alternate abbreviation of microRNA 410, as it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while retaining the same number.",
+"reason": "MIRN410 is an alternate abbreviation of microRNA 410, as it uses 'MIRN' instead of 'MIR' but still represents the same gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18780,7 +18778,7 @@
       <c r="L219" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'mir-491' is a lowercase version of the primary gene symbol 'MIR491' and represents the same microRNA gene.",
+"reason": "The alias symbol 'mir-491' is a lowercase version of the primary gene symbol 'MIR491', representing the same microRNA gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18949,7 +18947,7 @@
       <c r="L221" t="inlineStr">
         <is>
           <t>{
-"reason": "RanBP2L2 is not an alternate abbreviation of the official gene name because it represents a different description of the gene (RANBP2 like) without including the GRIP domain or the number 6.",
+"reason": "RanBP2L2 is not an alternate abbreviation because it represents a different description of the gene (RANBP2 like) rather than an abbreviation of the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -19204,7 +19202,7 @@
       <c r="L224" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol SNORA25A is not an alternate abbreviation because it contains an additional 'A' character that is not present in the official gene name or primary symbol.",
+"reason": "The alias symbol SNORA25A is not an alternate abbreviation because it includes an additional 'A' character that is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -19963,7 +19961,7 @@
       <c r="L233" t="inlineStr">
         <is>
           <t>{
-"reason": "ELA1 is an alternate abbreviation of the official gene name 'chymotrypsin like elastase 1' as it uses the first letter of 'elastase' and '1' from the name.",
+"reason": "ELA1 is an alternate abbreviation of the official gene name 'chymotrypsin like elastase 1' as it uses the first letter of 'elastase' and the number '1' from the full name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20132,7 +20130,7 @@
       <c r="L235" t="inlineStr">
         <is>
           <t>{
-"reason": "CT45-4 is not an alternate abbreviation because it represents a different member of the CT45 family (CT45-4) rather than the specific gene CT45A5.",
+"reason": "CT45-4 is not an alternate abbreviation because it represents a different member of the CT45 family (CT45-4) compared to the official gene (CT45A5).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -20725,7 +20723,7 @@
       <c r="L242" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'tRNA-Ala-AGC-13-1' is an expanded version of the official gene name 'tRNA-Ala (anticodon AGC) 13-1', containing the same information in a slightly different format.",
+"reason": "The alias symbol 'tRNA-Ala-AGC-13-1' is an expanded version of the official gene name 'tRNA-Ala (anticodon AGC) 13-1', using the same components in a slightly different format.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20811,7 +20809,7 @@
       <c r="L243" t="inlineStr">
         <is>
           <t>{
-"reason": "TRNAD18 is not an alternate abbreviation of the official gene name 'tRNA-Asp (anticodon GTC) 2-1' as it contains characters (18) not present in the official name and does not represent the same gene description.",
+"reason": "TRNAD18 is not an alternate abbreviation of the official gene name 'tRNA-Asp (anticodon GTC) 2-1' as it contains characters (18) not present in the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -20897,7 +20895,7 @@
       <c r="L244" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'nmt-tRNA-Gln-TTG-7-1' is an expanded version of the primary gene symbol 'NMTRQ-TTG7-1', representing the same gene with a more descriptive format that matches the official gene name.",
+"reason": "The alias symbol 'nmt-tRNA-Gln-TTG-7-1' is an expanded version of the primary gene symbol 'NMTRQ-TTG7-1', representing the same gene with a more descriptive abbreviation that matches the official gene name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -21069,7 +21067,7 @@
       <c r="L246" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN1185-1 is an alternate abbreviation of microRNA 1185-1 because it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while maintaining the same numeric identifier.",
+"reason": "MIRN1185-1 is an alternate abbreviation of microRNA 1185-1 because it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while maintaining the same numerical identifier.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -21155,8 +21153,8 @@
       <c r="L247" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol HSA-MIR-548H-1 is not an alternate abbreviation because it contains additional characters (HSA- and -) that are not present in the official gene name or primary symbol.",
-"alternate_abbreviation": "FALSE"
+"reason": "The alias symbol HSA-MIR-548H-1 is an alternate abbreviation of the official gene name 'microRNA 548h-1' with added hyphens and 'HSA' prefix.",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -21410,7 +21408,7 @@
       <c r="L250" t="inlineStr">
         <is>
           <t>{
-"reason": "FAT is not an alternate abbreviation because it is a shortened version of the primary gene symbol FAT1, which likely represents a gene family name rather than an abbreviation variant of the specific gene.",
+"reason": "FAT is not an alternate abbreviation because it is a shortened version of the primary gene symbol FAT1, likely representing a family name rather than a specific gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21748,7 +21746,7 @@
       <c r="L254" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L26 pseudogene 30'.",
+"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, making it not an alternate abbreviation.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21917,7 +21915,7 @@
       <c r="L256" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL39_3_134 contains additional characters (_3_134) not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L39 pseudogene 11'.",
+"reason": "The alias symbol RPL39_3_134 contains additional characters (_3_134) that are not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L39 pseudogene 11'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22086,7 +22084,7 @@
       <c r="L258" t="inlineStr">
         <is>
           <t>{
-"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because it represents a different member of the FKBP family (FKBP9 vs FKBP1B).",
+"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because it contains a different number (9) than the primary gene symbol (1B), indicating it likely represents a different gene in the same family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22341,7 +22339,7 @@
       <c r="L261" t="inlineStr">
         <is>
           <t>{
-"reason": "FRgamma is an alternate abbreviation as it represents 'folate receptor gamma' using different letters (FR) than the primary symbol (FOLR3).",
+"reason": "FRgamma is an alternate abbreviation as it represents 'folate receptor gamma' using different letters than the primary symbol FOLR3.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -22845,7 +22843,7 @@
       <c r="L267" t="inlineStr">
         <is>
           <t>{
-"reason": "TH2-LCR is an alternate abbreviation of the official gene name as it represents the same concept with a hyphen instead of the word 'associated' and 'RNA'.",
+"reason": "TH2-LCR is an alternate abbreviation of the official gene name as it represents the same concept with a hyphen added for readability.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -23595,7 +23593,7 @@
       <c r="L276" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol DDX3YP1 contains a 'Y' that is not present in the official gene name or primary symbol, indicating it likely represents a different gene or variant.",
+"reason": "The alias symbol DDX3YP1 contains a 'Y' that is not present in the official gene name or primary symbol, indicating it likely refers to a different gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -23850,7 +23848,7 @@
       <c r="L279" t="inlineStr">
         <is>
           <t>{
-"reason": "RN5S434 is an alternate abbreviation of RNA, 5S ribosomal pseudogene 434 as it uses different letters to represent the same gene name components.",
+"reason": "RN5S434 is an alternate abbreviation of RNA5SP434 as it represents the same gene with a shortened form of the primary symbol.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -24941,7 +24939,7 @@
       <c r="L292" t="inlineStr">
         <is>
           <t>{
-"reason": "SCHAD is not derived from the letters in the official gene name 'hydroxysteroid 17-beta dehydrogenase 10' or the primary symbol 'HSD17B10'.",
+"reason": "SCHAD is not derived from the letters in the official gene name 'hydroxysteroid 17-beta dehydrogenase 10' or the primary symbol 'HSD17B10', suggesting it represents a different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25362,7 +25360,7 @@
       <c r="L297" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'onco-lncRNA-32' is not an abbreviation variant of the official gene name as it includes additional information ('onco') and a different number ('32') not present in the official name.",
+"reason": "The alias symbol 'onco-lncRNA-32' is not an abbreviation variant of the official gene name as it includes additional descriptive elements ('onco' and '32') not present in the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25448,7 +25446,7 @@
       <c r="L298" t="inlineStr">
         <is>
           <t>{
-"reason": "A1B is a shortened version of the primary gene symbol A1BG, representing the same gene without altering the meaning.",
+"reason": "A1B is a shortened version of the primary gene symbol A1BG, representing the same gene without altering its meaning.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -26622,7 +26620,7 @@
       <c r="L312" t="inlineStr">
         <is>
           <t>{
-"reason": "V1-17 is not an alternate abbreviation of IGLV1-47 or immunoglobulin lambda variable 1-47 because it represents a different numbered variant of the gene family.",
+"reason": "V1-17 is not an alternate abbreviation of 'immunoglobulin lambda variable 1-47' as it represents a different numbered variant of the gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -26874,7 +26872,7 @@
       <c r="L315" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' with a hyphen added between IL and 12A.",
+"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' as it includes a hyphen between IL and 12A but represents the same gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -27885,7 +27883,7 @@
       <c r="L327" t="inlineStr">
         <is>
           <t>{
-"reason": "SAMS1 is not derived from the letters in the official gene name 'methionine adenosyltransferase 1A' or the primary symbol MAT1A, but appears to represent a different description of the gene's function.",
+"reason": "SAMS1 is not derived from the official gene name 'methionine adenosyltransferase 1A' or the primary symbol MAT1A, but likely stands for a different description of the gene's function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -28386,7 +28384,7 @@
       <c r="L333" t="inlineStr">
         <is>
           <t>{
-"reason": "MOCS1P2 is not an alternate abbreviation of MOCS1P1 or 'molybdenum cofactor synthesis 1 pseudogene 1' because it represents a different pseudogene number (2 instead of 1).",
+"reason": "MOCS1P2 is not an alternate abbreviation of MOCS1P1 or the official gene name because it represents a different pseudogene (2 instead of 1) in the same gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29234,7 +29232,7 @@
       <c r="L343" t="inlineStr">
         <is>
           <t>{
-"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains an 'L' which is not present in the official name or primary symbol.",
+"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains characters (L and 211) that are not present in the official name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30322,7 +30320,7 @@
       <c r="L356" t="inlineStr">
         <is>
           <t>{
-"reason": "Pr1/Pr2 is not an alternate abbreviation of 'proline rich protein HaeIII subfamily 1' as it represents different subfamily members (1 and 2) rather than an abbreviation of the official gene name.",
+"reason": "Pr1/Pr2 is not an alternate abbreviation of the official gene name as it represents different gene numbers (1 and 2) compared to the primary symbol PRH1.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30657,7 +30655,7 @@
       <c r="L360" t="inlineStr">
         <is>
           <t>{
-"reason": "SPF27 is not derived from the official gene name 'BCAS2 pre-mRNA processing factor' and appears to represent a different description of the gene.",
+"reason": "SPF27 is not derived from the letters in the official gene name 'BCAS2 pre-mRNA processing factor' and appears to represent a different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30909,7 +30907,7 @@
       <c r="L363" t="inlineStr">
         <is>
           <t>{
-"reason": "HNRNP-G is not an abbreviation variant of 'RBMX pseudogene 1' or 'RBMXP1', as it represents a different description of the gene (heterogeneous nuclear ribonucleoprotein G) rather than an alternate abbreviation of the official name.",
+"reason": "HNRNP-G is not an abbreviation variant of RBMX pseudogene 1 or RBMXP1, as it represents a different description of the gene (heterogeneous nuclear ribonucleoprotein G) rather than an alternate abbreviation of the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -31078,8 +31076,8 @@
       <c r="L365" t="inlineStr">
         <is>
           <t>{
-"reason": "RECC1 is an alternate abbreviation for 'replication factor C subunit 1' using different letters to represent the same concept as RFC1.",
-"alternate_abbreviation": "TRUE"
+"reason": "RECC1 is not an alternate abbreviation of 'replication factor C subunit 1' as it contains a 'C' not present in the official gene name.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>

</xml_diff>

<commit_message>
added a preprocessing exclusion step- "hsa-"prefix. 86%P 96%R
</commit_message>
<xml_diff>
--- a/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
+++ b/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
@@ -656,7 +656,7 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RN7SL427P is not an alternate abbreviation of the official gene name because it contains the number '427' which is not present in the official gene name or primary symbol.",
+"reason": "The alias symbol RN7SL427P is not an alternate abbreviation of the official gene name because it contains the number 427, which is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -825,7 +825,7 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>{
-"reason": "U51 is not an alternate abbreviation of the official gene name or primary symbol, as it represents a different description or classification of the gene.",
+"reason": "U51 is not an alternate abbreviation of the official gene name as it does not represent the same description using different letters.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -911,7 +911,7 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>{
-"reason": "RPL36A is not an alternate abbreviation of 'ribosomal protein L36a like' because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
+"reason": "RPL36A is not an alternate abbreviation because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1332,7 +1332,7 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>{
-"reason": "HOCT1 is not derived from the letters in the official gene name 'solute carrier family 22 member 1' or the primary symbol SLC22A1, but rather appears to be a different description or acronym for the gene.",
+"reason": "HOCT1 is not derived from the letters in the official gene name 'solute carrier family 22 member 1' or the primary symbol SLC22A1, but appears to be a different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1922,7 +1922,7 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>{
-"reason": "TRBF2 is an alternate abbreviation of 'telomeric repeat binding factor 2' using different letters to represent the same concept as TERF2.",
+"reason": "TRBF2 is an alternate abbreviation of 'telomeric repeat binding factor 2' using different letters to represent the same concept.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2008,7 +2008,7 @@
       <c r="L19" t="inlineStr">
         <is>
           <t>{
-"reason": "TGFR-1 is an alternate abbreviation of the official gene name as it represents 'transforming growth factor receptor 1' with a different letter arrangement.",
+"reason": "TGFR-1 is an alternate abbreviation of the official gene name as it represents 'transforming growth factor receptor 1' using different letters but maintaining the same meaning.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2343,7 +2343,7 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>{
-"reason": "TCRBV11S3 is an alternate abbreviation of the official gene name as it represents the same T cell receptor beta variable gene with a slightly different numbering format.",
+"reason": "TCRBV11S3 is an alternate abbreviation of 'T cell receptor beta variable 11-3' as it uses different letters to represent the same gene name components.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2927,7 +2927,7 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>{
-"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene but with the 'H' omitted from the primary symbol.",
+"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene name but with one letter omitted.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -3597,7 +3597,7 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>{
-"reason": "RI58 does not appear to be derived from the letters in the official gene name or primary symbol IFIT5.",
+"reason": "RI58 does not appear to be derived from the official gene name or primary symbol IFIT5, and likely represents a different description or naming convention for the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -3683,7 +3683,7 @@
       <c r="L39" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'Ly-6D' is an alternate abbreviation of the primary gene symbol 'LY6D' with only a minor difference in capitalization and hyphenation.",
+"reason": "The alias symbol 'Ly-6D' is an alternate abbreviation of the primary gene symbol 'LY6D', differing only in the use of a hyphen and lowercase 'y'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -4522,7 +4522,7 @@
       <c r="L49" t="inlineStr">
         <is>
           <t>{
-"reason": "CLEC4N is not an alternate abbreviation of the official gene name as it contains a different number (4) than the primary gene symbol (6), indicating it likely represents a different member of the CLEC family.",
+"reason": "CLEC4N is not an alternate abbreviation of the official gene name 'C-type lectin domain containing 6A' as it contains a different number (4) than the primary symbol (6).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4608,7 +4608,7 @@
       <c r="L50" t="inlineStr">
         <is>
           <t>{
-"reason": "DECTIN1 is not an alternate abbreviation of the official gene name 'C-type lectin domain containing 7A' as it represents a different description of the gene function.",
+"reason": "DECTIN1 is not derived from the official gene name 'C-type lectin domain containing 7A' or the primary symbol CLEC7A, but represents a different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4694,7 +4694,7 @@
       <c r="L51" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol OR10AC1P is not an alternate abbreviation because it includes an additional 'P' at the end, which is not present in the official gene name or primary symbol and likely indicates a pseudogene variant.",
+"reason": "The alias symbol OR10AC1P is not an alternate abbreviation because it includes a 'P' at the end, which is not present in the official gene name and likely indicates a pseudogene variant.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4780,7 +4780,7 @@
       <c r="L52" t="inlineStr">
         <is>
           <t>{
-"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, as it uses 'H' instead of 'L' but still represents the same gene concept.",
+"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, where 'H' likely stands for 'homolog' or 'human', which is not present in the official gene name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -5619,7 +5619,7 @@
       <c r="L62" t="inlineStr">
         <is>
           <t>{
-"reason": "UNCL is not an alternate abbreviation of the official gene name as it lacks the number '50' which is present in the primary gene symbol UNC50.",
+"reason": "UNCL is not an alternate abbreviation because it represents a different description or variant of the gene, not just a different way to abbreviate the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6292,7 +6292,7 @@
       <c r="L70" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '4E-T' is an abbreviated form of 'eIF4E transporter' which is not present in the official gene name, so it is not an alternate abbreviation of the official name.",
+"reason": "The alias symbol '4E-T' is not derived from the letters in the official gene name, but rather represents a different description of the gene's function.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6630,7 +6630,7 @@
       <c r="L74" t="inlineStr">
         <is>
           <t>{
-"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' or CNMD, as it appears to be derived from a different description of the gene.",
+"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' or CNMD as it contains letters not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -7392,7 +7392,7 @@
       <c r="L83" t="inlineStr">
         <is>
           <t>{
-"reason": "ACT is not an alternate abbreviation of 'actin beta like 2' as it does not include the 'beta like 2' part of the official gene name.",
+"reason": "ACT is not an alternate abbreviation of 'actin beta like 2' as it does not include the 'BL2' component which represents 'beta like 2' in the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -8145,7 +8145,7 @@
       <c r="L92" t="inlineStr">
         <is>
           <t>{
-"reason": "A4GALT1 is not an alternate abbreviation because it includes an additional '1' that is not present in the official gene name or primary gene symbol.",
+"reason": "A4GALT1 is not an alternate abbreviation because it includes an additional '1' at the end, which is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -8898,7 +8898,7 @@
       <c r="L101" t="inlineStr">
         <is>
           <t>{
-"reason": "SNAT is an alternate abbreviation of the official gene name 'aralkylamine N-acetyltransferase' as it uses different letters to represent the same concept.",
+"reason": "SNAT is an alternate abbreviation of the official gene name 'aralkylamine N-acetyltransferase' as it uses different letters to represent the same enzyme.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -9568,8 +9568,8 @@
       <c r="L109" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol HMGB1L14 is not an alternate abbreviation because it uses 'L' instead of 'P' to represent 'pseudogene', which is not consistent with the official gene name.",
-"alternate_abbreviation": "FALSE"
+"reason": "The alias symbol HMGB1L14 is an alternate abbreviation of the official gene name, replacing 'pseudogene' with 'L' while maintaining the same meaning and number.",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -10733,7 +10733,7 @@
       <c r="L123" t="inlineStr">
         <is>
           <t>{
-"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and appears to represent a different aspect of the gene.",
+"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and likely represents a different aspect of the gene's function or characteristics.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12066,7 +12066,7 @@
       <c r="L139" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '#NAME?' is not a valid gene symbol and does not appear to be an abbreviation variant of the official gene name 'mediator complex subunit 23' or the primary symbol 'MED23'.",
+"reason": "The alias symbol '#NAME?' does not appear to be an abbreviation variant of the official gene name 'mediator complex subunit 23' or the primary symbol 'MED23'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12404,7 +12404,7 @@
       <c r="L143" t="inlineStr">
         <is>
           <t>{
-"reason": "ACF is an alternate abbreviation of the official gene name 'APOBEC1 complementation factor' as it uses the first letter of each word in the name.",
+"reason": "ACF is an alternate abbreviation of the official gene name APOBEC1 complementation factor, using the first letter of each word.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -12659,7 +12659,7 @@
       <c r="L146" t="inlineStr">
         <is>
           <t>{
-"reason": "CPX-IV is an alternate abbreviation of complexin 4, using 'CPX' instead of 'CPLX' and Roman numeral 'IV' instead of '4'.",
+"reason": "CPX-IV is an alternate abbreviation of complexin 4, using 'CPX' for 'complexin' and 'IV' (Roman numeral) for '4'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -14909,7 +14909,7 @@
       <c r="L173" t="inlineStr">
         <is>
           <t>{
-"reason": "PCN3 is not derived from the letters in the official gene name 'cytochrome P450 family 3 subfamily A member 5' or the primary symbol CYP3A5.",
+"reason": "PCN3 is not derived from the official gene name or primary symbol and appears to represent a different description or aspect of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -15164,7 +15164,7 @@
       <c r="L176" t="inlineStr">
         <is>
           <t>{
-"reason": "EFO2p is not an alternate abbreviation of ESCO2 or the official gene name, as it contains a 'p' which is not present in either the primary symbol or the official name.",
+"reason": "EFO2p is not an alternate abbreviation of ESCO2 or the official gene name as it contains a 'p' which is not present in either the primary symbol or the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -15499,7 +15499,7 @@
       <c r="L180" t="inlineStr">
         <is>
           <t>{
-"reason": "CSTF3-AS1 is not an alternate abbreviation because it represents a different description of the gene (antisense RNA) compared to the official gene name (divergent transcript).",
+"reason": "The alias symbol CSTF3-AS1 is not an alternate abbreviation of the official gene name 'CSTF3 divergent transcript' as it represents a different description (antisense RNA) rather than an abbreviation variant.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -18179,7 +18179,7 @@
       <c r="L212" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN139 is an alternate abbreviation of microRNA 139, as it uses 'MIRN' instead of 'MIR' to represent 'microRNA'.",
+"reason": "MIRN139 is an alternate abbreviation of microRNA 139, as it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while retaining the same number.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18351,7 +18351,7 @@
       <c r="L214" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'A' at the end.",
+"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'a' at the end.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18778,7 +18778,7 @@
       <c r="L219" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'mir-491' is a lowercase version of the primary gene symbol 'MIR491', representing the same microRNA gene.",
+"reason": "The alias symbol 'mir-491' is a lowercase version of the primary gene symbol 'MIR491' and represents the same microRNA gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -19457,7 +19457,7 @@
       <c r="L227" t="inlineStr">
         <is>
           <t>{
-"reason": "ACA36b is an alternate abbreviation of the official gene name as it represents 'H/ACA box 36B' from the full name.",
+"reason": "ACA36b is an alternate abbreviation of the official gene name as it represents 'H/ACA box 36B' from the full name 'small nucleolar RNA, H/ACA box 36B'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -19961,7 +19961,7 @@
       <c r="L233" t="inlineStr">
         <is>
           <t>{
-"reason": "ELA1 is an alternate abbreviation of the official gene name 'chymotrypsin like elastase 1' as it uses the first letter of 'elastase' and the number '1' from the full name.",
+"reason": "ELA1 is an alternate abbreviation of CELA1 as it represents the same gene (chymotrypsin like elastase 1) using different letters.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20809,7 +20809,7 @@
       <c r="L243" t="inlineStr">
         <is>
           <t>{
-"reason": "TRNAD18 is not an alternate abbreviation of the official gene name 'tRNA-Asp (anticodon GTC) 2-1' as it contains characters (18) not present in the official name.",
+"reason": "TRNAD18 is not an alternate abbreviation of the official gene name 'tRNA-Asp (anticodon GTC) 2-1' as it contains characters (18) not present in the official name and does not represent the same gene description.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21067,7 +21067,7 @@
       <c r="L246" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN1185-1 is an alternate abbreviation of microRNA 1185-1 because it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while maintaining the same numerical identifier.",
+"reason": "MIRN1185-1 is an alternate abbreviation of microRNA 1185-1 as it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while maintaining the same numerical identifier.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -21746,7 +21746,7 @@
       <c r="L254" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, making it not an alternate abbreviation.",
+"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L26 pseudogene 30'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21915,7 +21915,7 @@
       <c r="L256" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL39_3_134 contains additional characters (_3_134) that are not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L39 pseudogene 11'.",
+"reason": "The alias symbol RPL39_3_134 is not an alternate abbreviation because it contains additional characters (_3_134) that are not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22084,7 +22084,7 @@
       <c r="L258" t="inlineStr">
         <is>
           <t>{
-"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because it contains a different number (9) than the primary gene symbol (1B), indicating it likely represents a different gene in the same family.",
+"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because it represents a different member of the FKBP family (FKBP9 vs FKBP1B).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22170,7 +22170,7 @@
       <c r="L259" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol TRIM49D2P is not an alternate abbreviation because it contains an additional 'P' character not present in the official gene name or primary symbol.",
+"reason": "The alias symbol TRIM49D2P is not an alternate abbreviation because it contains an additional 'P' character that is not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22508,7 +22508,7 @@
       <c r="L263" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'mir-3151' is an alternate abbreviation of the official gene name 'microRNA 3151' as it represents the same gene with a slight variation in capitalization and hyphenation.",
+"reason": "The alias symbol 'mir-3151' is a lowercase version of the primary gene symbol 'MIR3151', representing the same microRNA.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -22843,7 +22843,7 @@
       <c r="L267" t="inlineStr">
         <is>
           <t>{
-"reason": "TH2-LCR is an alternate abbreviation of the official gene name as it represents the same concept with a hyphen added for readability.",
+"reason": "TH2-LCR is an alternate abbreviation of the official gene name as it represents the same concept with a hyphen instead of the word 'associated' and 'RNA'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -23593,7 +23593,7 @@
       <c r="L276" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol DDX3YP1 contains a 'Y' that is not present in the official gene name or primary symbol, indicating it likely refers to a different gene.",
+"reason": "The alias symbol DDX3YP1 is not an alternate abbreviation because it contains a 'Y' character that is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25360,7 +25360,7 @@
       <c r="L297" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'onco-lncRNA-32' is not an abbreviation variant of the official gene name as it includes additional descriptive elements ('onco' and '32') not present in the official name.",
+"reason": "The alias symbol 'onco-lncRNA-32' is not an alternate abbreviation of the official gene name as it includes additional descriptive elements ('onco' and '32') not present in the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25446,7 +25446,7 @@
       <c r="L298" t="inlineStr">
         <is>
           <t>{
-"reason": "A1B is a shortened version of the primary gene symbol A1BG, representing the same gene without altering its meaning.",
+"reason": "A1B is a shortened version of the primary gene symbol A1BG and represents the same gene without introducing new characters.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -26872,7 +26872,7 @@
       <c r="L315" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' as it includes a hyphen between IL and 12A but represents the same gene.",
+"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' with a hyphen added between IL and 12A.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -27041,7 +27041,7 @@
       <c r="L317" t="inlineStr">
         <is>
           <t>{
-"reason": "ITGB1BP is not an alternate abbreviation because it is a shortened version of the primary gene symbol ITGB1BP2, likely representing a family name rather than the specific gene.",
+"reason": "The alias symbol ITGB1BP is not an alternate abbreviation because it lacks the number '2' present in the primary gene symbol ITGB1BP2, which indicates it may represent a different gene or gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -27382,7 +27382,7 @@
       <c r="L321" t="inlineStr">
         <is>
           <t>{
-"reason": "IPOA7 is an alternate abbreviation for 'importin alpha 7', which is a previous name for karyopherin subunit alpha 6.",
+"reason": "IPOA7 is an alternate abbreviation for 'importin alpha 7', which is a previous name for karyopherin subunit alpha 6, representing the same gene with different terminology.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -27883,7 +27883,7 @@
       <c r="L327" t="inlineStr">
         <is>
           <t>{
-"reason": "SAMS1 is not derived from the official gene name 'methionine adenosyltransferase 1A' or the primary symbol MAT1A, but likely stands for a different description of the gene's function.",
+"reason": "SAMS1 is not an alternate abbreviation of 'methionine adenosyltransferase 1A' as it represents a different description of the gene (S-adenosylmethionine synthetase 1) rather than a variant abbreviation of the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -28384,7 +28384,7 @@
       <c r="L333" t="inlineStr">
         <is>
           <t>{
-"reason": "MOCS1P2 is not an alternate abbreviation of MOCS1P1 or the official gene name because it represents a different pseudogene (2 instead of 1) in the same gene family.",
+"reason": "MOCS1P2 is not an alternate abbreviation of MOCS1P1 or the official gene name because it represents a different pseudogene (P2 instead of P1) in the same gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29060,7 +29060,7 @@
       <c r="L341" t="inlineStr">
         <is>
           <t>{
-"reason": "GCNF1 is not an alternate abbreviation of the official gene name as it represents a different description (Germ Cell Nuclear Factor 1) rather than an abbreviation of 'nuclear receptor subfamily 6 group A member 1'.",
+"reason": "GCNF1 is not an alternate abbreviation of the official gene name as it represents a different description (Germ Cell Nuclear Factor) rather than an abbreviation of 'nuclear receptor subfamily 6 group A member 1'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29232,7 +29232,7 @@
       <c r="L343" t="inlineStr">
         <is>
           <t>{
-"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains characters (L and 211) that are not present in the official name or primary symbol.",
+"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains characters (L and 211) not present in 'olfactory receptor family 1 subfamily C member 1'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30320,7 +30320,7 @@
       <c r="L356" t="inlineStr">
         <is>
           <t>{
-"reason": "Pr1/Pr2 is not an alternate abbreviation of the official gene name as it represents different gene numbers (1 and 2) compared to the primary symbol PRH1.",
+"reason": "Pr1/Pr2 is not an alternate abbreviation of 'proline rich protein HaeIII subfamily 1' as it represents different subfamily members (1 and 2) rather than the specific PRH1 gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30655,7 +30655,7 @@
       <c r="L360" t="inlineStr">
         <is>
           <t>{
-"reason": "SPF27 is not derived from the letters in the official gene name 'BCAS2 pre-mRNA processing factor' and appears to represent a different description of the gene.",
+"reason": "SPF27 is not derived from the official gene name 'BCAS2 pre-mRNA processing factor' and appears to represent a different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>

</xml_diff>

<commit_message>
added a bit about if the symbol represents a previous name it is not an alternate abbrev. 89%P 91%R
</commit_message>
<xml_diff>
--- a/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
+++ b/output/consolidated_alt_abbrev_annotation_with_prompt_no_context_df.xlsx
@@ -529,7 +529,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -615,7 +615,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -701,7 +701,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -784,7 +784,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -825,7 +825,7 @@
       <c r="L5" t="inlineStr">
         <is>
           <t>{
-"reason": "U51 is not an alternate abbreviation of the official gene name as it does not represent the same description using different letters.",
+"reason": "U51 is not an alternate abbreviation of 'small nucleolar RNA, C/D box 51' as it does not represent the same name using different letters.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -870,7 +870,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -911,7 +911,7 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>{
-"reason": "RPL36A is not an alternate abbreviation because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
+"reason": "RPL36A is not an alternate abbreviation of 'ribosomal protein L36a like' because it lacks the 'L' at the end, which stands for 'like' in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -956,7 +956,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1039,7 +1039,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1122,7 +1122,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1163,7 +1163,7 @@
       <c r="L9" t="inlineStr">
         <is>
           <t>{
-"reason": "MCT3 is an alternate abbreviation for 'monocarboxylate transporter 3', which is a different description of the gene and not directly related to the official name 'solute carrier family 16 member 3'.",
+"reason": "MCT3 is not an alternate abbreviation of the official gene name 'solute carrier family 16 member 3' as it represents a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1208,7 +1208,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1291,7 +1291,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1332,7 +1332,7 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>{
-"reason": "HOCT1 is not derived from the letters in the official gene name 'solute carrier family 22 member 1' or the primary symbol SLC22A1, but appears to be a different description of the gene.",
+"reason": "HOCT1 is not an alternate abbreviation of the official gene name 'solute carrier family 22 member 1' as it represents a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1377,7 +1377,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1418,7 +1418,7 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>{
-"reason": "ARALAR1 is not derived from the official gene name 'solute carrier family 25 member 12' or the primary symbol SLC25A12, but appears to be a different description or name for the gene.",
+"reason": "ARALAR1 is not an abbreviation variant of 'solute carrier family 25 member 12' as it represents a different name or description of the gene rather than an alternate abbreviation of the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -1463,7 +1463,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1546,7 +1546,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1632,7 +1632,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1715,7 +1715,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1798,7 +1798,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1881,7 +1881,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -1922,7 +1922,7 @@
       <c r="L18" t="inlineStr">
         <is>
           <t>{
-"reason": "TRBF2 is an alternate abbreviation of 'telomeric repeat binding factor 2' using different letters to represent the same concept.",
+"reason": "TRBF2 is an alternate abbreviation of the official gene name 'telomeric repeat binding factor 2' as it uses the first letters of each word in the name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -1967,7 +1967,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2053,7 +2053,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2136,7 +2136,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2219,7 +2219,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2302,7 +2302,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2343,7 +2343,7 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>{
-"reason": "TCRBV11S3 is an alternate abbreviation of 'T cell receptor beta variable 11-3' as it uses different letters to represent the same gene name components.",
+"reason": "TCRBV11S3 is an alternate abbreviation of T cell receptor beta variable 11-3, using 'C' for 'cell' and 'S' instead of '-'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2388,7 +2388,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2471,7 +2471,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2554,7 +2554,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2637,7 +2637,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2720,7 +2720,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2803,7 +2803,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2886,7 +2886,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -2927,7 +2927,7 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>{
-"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene name but with one letter omitted.",
+"reason": "URF2 is an alternate abbreviation of UHRF2, as it represents the same gene name but with the 'H' omitted.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -2972,7 +2972,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3055,7 +3055,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3138,7 +3138,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3179,7 +3179,7 @@
       <c r="L33" t="inlineStr">
         <is>
           <t>{
-"reason": "SMARCM1 is not derived from the official gene name 'BCL11 transcription factor A' or the primary symbol 'BCL11A', and appears to represent a different description of the gene.",
+"reason": "SMARCM1 is not derived from the letters in the official gene name 'BCL11 transcription factor A' or the primary symbol 'BCL11A', so it is not an alternate abbreviation.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -3224,7 +3224,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3307,7 +3307,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3390,7 +3390,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3473,7 +3473,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3556,7 +3556,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3597,7 +3597,7 @@
       <c r="L38" t="inlineStr">
         <is>
           <t>{
-"reason": "RI58 does not appear to be derived from the official gene name or primary symbol IFIT5, and likely represents a different description or naming convention for the gene.",
+"reason": "RI58 is not derived from the letters in the official gene name or primary symbol IFIT5, so it is not an alternate abbreviation.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -3642,7 +3642,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3683,7 +3683,7 @@
       <c r="L39" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'Ly-6D' is an alternate abbreviation of the primary gene symbol 'LY6D', differing only in the use of a hyphen and lowercase 'y'.",
+"reason": "The alias symbol 'Ly-6D' is an alternate abbreviation of the primary gene symbol 'LY6D' with a hyphen added between 'Ly' and '6D'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -3728,7 +3728,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3811,7 +3811,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3894,7 +3894,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -3935,7 +3935,7 @@
       <c r="L42" t="inlineStr">
         <is>
           <t>{
-"reason": "CALS is not an alternate abbreviation of 'carbonic anhydrase 8' as it contains letters not present in the official gene name.",
+"reason": "CALS is not an alternate abbreviation of 'carbonic anhydrase 8 (inactive)' as it contains letters not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -3980,7 +3980,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4063,7 +4063,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4146,7 +4146,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4229,7 +4229,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4312,7 +4312,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4395,7 +4395,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4436,7 +4436,7 @@
       <c r="L48" t="inlineStr">
         <is>
           <t>{
-"reason": "MS22 is an alternate abbreviation of MRPS22 as it represents the same gene name (mitochondrial ribosomal protein S22) with fewer letters.",
+"reason": "MS22 is an alternate abbreviation of MRPS22 as it represents the same gene name (mitochondrial ribosomal protein S22) but with fewer letters.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -4481,7 +4481,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4522,7 +4522,7 @@
       <c r="L49" t="inlineStr">
         <is>
           <t>{
-"reason": "CLEC4N is not an alternate abbreviation of the official gene name 'C-type lectin domain containing 6A' as it contains a different number (4) than the primary symbol (6).",
+"reason": "CLEC4N is not an alternate abbreviation of C-type lectin domain containing 6A because it contains a different number (4) than the primary gene symbol (6).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4567,7 +4567,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4608,7 +4608,7 @@
       <c r="L50" t="inlineStr">
         <is>
           <t>{
-"reason": "DECTIN1 is not derived from the official gene name 'C-type lectin domain containing 7A' or the primary symbol CLEC7A, but represents a different description of the gene.",
+"reason": "DECTIN1 is not an alternate abbreviation of the official gene name 'C-type lectin domain containing 7A' as it represents a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4653,7 +4653,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4739,7 +4739,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4780,8 +4780,8 @@
       <c r="L52" t="inlineStr">
         <is>
           <t>{
-"reason": "FCRH2 is an alternate abbreviation of Fc receptor like 2, where 'H' likely stands for 'homolog' or 'human', which is not present in the official gene name.",
-"alternate_abbreviation": "TRUE"
+"reason": "FCRH2 is not an alternate abbreviation of the official gene name 'Fc receptor like 2' as it contains an 'H' which is not present in the official name or primary symbol.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -4825,7 +4825,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4908,7 +4908,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -4949,7 +4949,7 @@
       <c r="L54" t="inlineStr">
         <is>
           <t>{
-"reason": "HHC is not derived from the letters in 'calcium sensing receptor' or 'CASR', so it is not an alternate abbreviation.",
+"reason": "HHC is not an alternate abbreviation of 'calcium sensing receptor' as it does not use letters from the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -4994,7 +4994,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5077,7 +5077,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5160,7 +5160,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5243,7 +5243,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5326,7 +5326,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5409,7 +5409,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5492,7 +5492,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5533,7 +5533,7 @@
       <c r="L61" t="inlineStr">
         <is>
           <t>{
-"reason": "SELOB is not derived from the letters in the official gene name or primary symbol SVEP1, and appears to represent a different description of the gene.",
+"reason": "SELOB is not derived from the letters in the official gene name or primary symbol SVEP1, and appears to represent a different description or previous name for the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -5578,7 +5578,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5619,7 +5619,7 @@
       <c r="L62" t="inlineStr">
         <is>
           <t>{
-"reason": "UNCL is not an alternate abbreviation because it represents a different description or variant of the gene, not just a different way to abbreviate the official gene name.",
+"reason": "UNCL is not an alternate abbreviation of the official gene name as it does not represent the same name with different letters, but rather appears to be a shortened form of the primary gene symbol UNC50.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -5664,7 +5664,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5705,7 +5705,7 @@
       <c r="L63" t="inlineStr">
         <is>
           <t>{
-"reason": "ACECS2L is not an alternate abbreviation of 'acyl-CoA synthetase short chain family member 1' as it contains additional characters (E, C, 2, L) not present in the official gene name.",
+"reason": "ACECS2L is not an alternate abbreviation of the official gene name as it contains characters (E and C) not present in the official name 'acyl-CoA synthetase short chain family member 1'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -5750,7 +5750,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5833,7 +5833,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -5916,7 +5916,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6002,7 +6002,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6085,7 +6085,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6168,7 +6168,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6251,7 +6251,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6292,7 +6292,7 @@
       <c r="L70" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '4E-T' is not derived from the letters in the official gene name, but rather represents a different description of the gene's function.",
+"reason": "The alias symbol '4E-T' is not derived from the letters in the official gene name, but rather appears to be a shorthand representation of a different description or function of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6337,7 +6337,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6420,7 +6420,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6461,7 +6461,7 @@
       <c r="L72" t="inlineStr">
         <is>
           <t>{
-"reason": "PDZD5A is not an alternate abbreviation of the official gene name as it only represents a part of the gene's function (PDZ domain) and does not include the FERM domain or indicate it's a pseudogene.",
+"reason": "PDZD5A is not an alternate abbreviation of FERM and PDZ domain containing 2B (pseudogene) as it represents a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6506,7 +6506,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6589,7 +6589,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6630,7 +6630,7 @@
       <c r="L74" t="inlineStr">
         <is>
           <t>{
-"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' or CNMD as it contains letters not present in the official gene name or primary symbol.",
+"reason": "CHM-I is not an alternate abbreviation of 'chondromodulin' or CNMD, but rather appears to be a previous name or different description of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6675,7 +6675,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6716,7 +6716,7 @@
       <c r="L75" t="inlineStr">
         <is>
           <t>{
-"reason": "DPB11 is not derived from the letters in the official gene name 'DNA topoisomerase II binding protein 1' or the primary symbol TOPBP1.",
+"reason": "DPB11 is not an alternate abbreviation of 'DNA topoisomerase II binding protein 1' as it contains letters not present in the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6761,7 +6761,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6844,7 +6844,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6885,7 +6885,7 @@
       <c r="L77" t="inlineStr">
         <is>
           <t>{
-"reason": "STIP-1 is not derived from the official gene name 'tuftelin interacting protein 11' or the primary symbol TFIP11, and appears to represent a different description of the gene.",
+"reason": "STIP-1 is not derived from the letters in the official gene name 'tuftelin interacting protein 11' or the primary symbol TFIP11, so it is not an alternate abbreviation.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -6930,7 +6930,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -6971,7 +6971,7 @@
       <c r="L78" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'hPot1' is an alternate abbreviation of the official gene name as it includes 'h' for human and capitalizes the first letter of 'Pot', while maintaining the same meaning.",
+"reason": "The alias symbol 'hPot1' is an alternate abbreviation of the official gene name 'protection of telomeres 1' as it includes the 'h' prefix for human and capitalizes the 'P' in 'Pot'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -7016,7 +7016,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7099,7 +7099,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7182,7 +7182,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7223,7 +7223,7 @@
       <c r="L81" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '82-FIP' does not appear to be derived from the official gene name 'nuclear FMR1 interacting protein 2' or the primary symbol 'NUFIP2', and contains numbers not present in either.",
+"reason": "The alias symbol '82-FIP' does not appear to be derived from the letters in the official gene name 'nuclear FMR1 interacting protein 2' or the primary symbol 'NUFIP2'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -7268,7 +7268,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7351,7 +7351,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7437,7 +7437,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7520,7 +7520,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7603,7 +7603,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7686,7 +7686,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7769,7 +7769,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7810,7 +7810,7 @@
       <c r="L88" t="inlineStr">
         <is>
           <t>{
-"reason": "ALPHA4GNT is an alternate abbreviation of the official gene name as it represents the same enzyme using 'ALPHA' instead of 'A' for 'alpha'.",
+"reason": "ALPHA4GNT is an alternate abbreviation of the official gene name as it represents the same meaning using different letters, with 'ALPHA' spelled out instead of abbreviated as 'A'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -7855,7 +7855,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -7938,7 +7938,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8021,7 +8021,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8104,7 +8104,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8145,7 +8145,7 @@
       <c r="L92" t="inlineStr">
         <is>
           <t>{
-"reason": "A4GALT1 is not an alternate abbreviation because it includes an additional '1' at the end, which is not present in the official gene name or primary symbol.",
+"reason": "The alias symbol A4GALT1 is not an alternate abbreviation because it includes an additional '1' at the end, which is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -8190,7 +8190,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8273,7 +8273,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8356,7 +8356,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8439,7 +8439,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8522,7 +8522,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8605,7 +8605,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8688,7 +8688,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8771,7 +8771,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8857,7 +8857,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -8943,7 +8943,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9026,7 +9026,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9109,7 +9109,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9192,7 +9192,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9275,7 +9275,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9358,7 +9358,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9441,7 +9441,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9527,7 +9527,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9568,8 +9568,8 @@
       <c r="L109" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol HMGB1L14 is an alternate abbreviation of the official gene name, replacing 'pseudogene' with 'L' while maintaining the same meaning and number.",
-"alternate_abbreviation": "TRUE"
+"reason": "The alias symbol HMGB1L14 is not an alternate abbreviation because it uses 'L' instead of 'P' to represent 'pseudogene', which is not consistent with the official gene name.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -9613,7 +9613,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9696,7 +9696,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9779,7 +9779,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9862,7 +9862,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -9945,7 +9945,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10028,7 +10028,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10111,7 +10111,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10194,7 +10194,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10277,7 +10277,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10360,7 +10360,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10443,7 +10443,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10526,7 +10526,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10609,7 +10609,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10692,7 +10692,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10733,7 +10733,7 @@
       <c r="L123" t="inlineStr">
         <is>
           <t>{
-"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', and likely represents a different aspect of the gene's function or characteristics.",
+"reason": "SMC is not derived from the letters in 'dymeclin' or 'DYM', so it is not an alternate abbreviation.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -10778,7 +10778,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10861,7 +10861,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -10944,7 +10944,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11027,7 +11027,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11110,7 +11110,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11193,7 +11193,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11276,7 +11276,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11359,7 +11359,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11442,7 +11442,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11483,7 +11483,7 @@
       <c r="L132" t="inlineStr">
         <is>
           <t>{
-"reason": "CPU is not an alternate abbreviation of carboxypeptidase B2 as it does not represent the same gene name using different letters.",
+"reason": "CPU is not an alternate abbreviation of carboxypeptidase B2 as it does not use letters from the official gene name in the same order.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -11528,7 +11528,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11611,7 +11611,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11694,7 +11694,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11780,7 +11780,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11863,7 +11863,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -11946,7 +11946,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12011,7 +12011,9 @@
           <t>MED23</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
+      <c r="E139" t="e">
+        <v>#NAME?</v>
+      </c>
       <c r="F139" t="inlineStr">
         <is>
           <t>mediator complex subunit 23</t>
@@ -12025,7 +12027,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12066,7 +12068,7 @@
       <c r="L139" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol '#NAME?' does not appear to be an abbreviation variant of the official gene name 'mediator complex subunit 23' or the primary symbol 'MED23'.",
+"reason": "The alias symbol '#NAME?' is not a valid gene symbol and does not appear to be an abbreviation variant of the official gene name 'mediator complex subunit 23' or the primary symbol 'MED23'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12111,7 +12113,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12194,7 +12196,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12277,7 +12279,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12318,7 +12320,7 @@
       <c r="L142" t="inlineStr">
         <is>
           <t>{
-"reason": "ARTC5 is an alternate abbreviation of ADP-ribosyltransferase 5, as it includes the 'C' from 'ribosyltransferase' in addition to the primary symbol ART5.",
+"reason": "ARTC5 is an alternate abbreviation of ADP-ribosyltransferase 5 as it includes the 'C' from 'ribosyltransferase' in addition to the primary symbol ART5.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -12363,7 +12365,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12449,7 +12451,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12532,7 +12534,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12573,7 +12575,7 @@
       <c r="L145" t="inlineStr">
         <is>
           <t>{
-"reason": "ASP is not derived from the letters in the official gene name 'APOBEC1 complementation factor' or the primary symbol 'A1CF'.",
+"reason": "ASP is not derived from the letters in the official gene name 'APOBEC1 complementation factor' or the primary symbol A1CF.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -12618,7 +12620,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12659,7 +12661,7 @@
       <c r="L146" t="inlineStr">
         <is>
           <t>{
-"reason": "CPX-IV is an alternate abbreviation of complexin 4, using 'CPX' for 'complexin' and 'IV' (Roman numeral) for '4'.",
+"reason": "CPX-IV is an alternate abbreviation of complexin 4, using 'CPX' for 'complexin' and 'IV' (Roman numeral 4) instead of '4'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -12704,7 +12706,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12787,7 +12789,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12873,7 +12875,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -12956,7 +12958,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13039,7 +13041,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13122,7 +13124,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13205,7 +13207,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13288,7 +13290,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13329,7 +13331,7 @@
       <c r="L154" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'pp75' does not appear to be derived from or related to the official gene name 'RAB11 family interacting protein 5' or the primary symbol 'RAB11FIP5'.",
+"reason": "The alias symbol 'pp75' does not appear to be derived from or related to the letters in the official gene name 'RAB11 family interacting protein 5' or the primary symbol 'RAB11FIP5'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -13374,7 +13376,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13457,7 +13459,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13540,7 +13542,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13623,7 +13625,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13706,7 +13708,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13789,7 +13791,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13872,7 +13874,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -13955,7 +13957,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14038,7 +14040,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14121,7 +14123,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14204,7 +14206,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14287,7 +14289,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14370,7 +14372,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14453,7 +14455,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14536,7 +14538,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14619,7 +14621,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14702,7 +14704,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14785,7 +14787,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14868,7 +14870,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14909,7 +14911,7 @@
       <c r="L173" t="inlineStr">
         <is>
           <t>{
-"reason": "PCN3 is not derived from the official gene name or primary symbol and appears to represent a different description or aspect of the gene.",
+"reason": "PCN3 is not derived from the letters in the official gene name 'cytochrome P450 family 3 subfamily A member 5' or the primary symbol CYP3A5.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -14954,7 +14956,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -14995,7 +14997,7 @@
       <c r="L174" t="inlineStr">
         <is>
           <t>{
-"reason": "FOR20 is not derived from the official gene name 'centrosomal protein 20' or the primary symbol CEP20, and appears to represent a different description of the gene.",
+"reason": "FOR20 is not an alternate abbreviation of 'centrosomal protein 20' as it uses different letters and represents a previous name (FOP-related protein of 20 kDa) rather than an abbreviation of the current official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -15040,7 +15042,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15123,7 +15125,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15164,7 +15166,7 @@
       <c r="L176" t="inlineStr">
         <is>
           <t>{
-"reason": "EFO2p is not an alternate abbreviation of ESCO2 or the official gene name as it contains a 'p' which is not present in either the primary symbol or the official name.",
+"reason": "EFO2p is not an alternate abbreviation of ESCO2 or the official gene name because it contains a 'p' which is not present in either the primary symbol or the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -15209,7 +15211,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15292,7 +15294,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15375,7 +15377,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15458,7 +15460,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15544,7 +15546,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15630,7 +15632,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15713,7 +15715,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15796,7 +15798,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15879,7 +15881,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -15962,7 +15964,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16003,7 +16005,7 @@
       <c r="L186" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'tamo' does not appear to be derived from or related to the official gene name 'spermatogenesis associated 2 like' or the primary symbol 'SPATA2L'.",
+"reason": "The alias symbol 'tamo' does not appear to be derived from or related to the letters in the official gene name 'spermatogenesis associated 2 like' or the primary symbol 'SPATA2L'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -16048,7 +16050,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16131,7 +16133,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16217,7 +16219,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16300,7 +16302,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16383,7 +16385,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16466,7 +16468,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16549,7 +16551,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16632,7 +16634,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16715,7 +16717,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16756,7 +16758,7 @@
       <c r="L195" t="inlineStr">
         <is>
           <t>{
-"reason": "EDA1R is not an alternate abbreviation of EDAR or 'ectodysplasin A receptor' as it contains a '1' which is not present in the official gene name or primary symbol.",
+"reason": "EDA1R is not an alternate abbreviation of EDAR or ectodysplasin A receptor as it contains the number '1' which is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -16801,7 +16803,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16884,7 +16886,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -16967,7 +16969,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17050,7 +17052,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17133,7 +17135,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17216,7 +17218,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17299,7 +17301,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17382,7 +17384,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17465,7 +17467,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17506,7 +17508,7 @@
       <c r="L204" t="inlineStr">
         <is>
           <t>{
-"reason": "RABJS is not an alternate abbreviation of the official gene name as it represents a different description of the gene (likely related to RAB proteins) rather than an abbreviation of 'DnaJ heat shock protein family (Hsp40) member C27'.",
+"reason": "RABJS is not an alternate abbreviation of the official gene name as it represents a different description or previous name of the gene, not a variant abbreviation of 'DnaJ heat shock protein family (Hsp40) member C27'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -17551,7 +17553,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17634,7 +17636,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17675,7 +17677,7 @@
       <c r="L206" t="inlineStr">
         <is>
           <t>{
-"reason": "TESSP1 is not an alternate abbreviation of 'serine protease 41' as it appears to represent a different description or aspect of the gene rather than an abbreviation of the official name.",
+"reason": "TESSP1 is not an alternate abbreviation of 'serine protease 41' as it appears to be a different name or previous designation for the gene rather than a variant abbreviation of the official name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -17720,7 +17722,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17803,7 +17805,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17886,7 +17888,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -17969,7 +17971,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18055,7 +18057,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18138,7 +18140,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18179,7 +18181,7 @@
       <c r="L212" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN139 is an alternate abbreviation of microRNA 139, as it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while retaining the same number.",
+"reason": "MIRN139 is an alternate abbreviation of microRNA 139, as it uses 'MIRN' instead of 'MIR' but still represents the same gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18224,7 +18226,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18310,7 +18312,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18351,7 +18353,7 @@
       <c r="L214" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'a' at the end.",
+"reason": "The alias symbol 'miR-20' is an abbreviated form of the official gene name 'microRNA 20a', omitting the 'A' at the end.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18396,7 +18398,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18437,7 +18439,7 @@
       <c r="L215" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN95 is an alternate abbreviation of microRNA 95, as it uses 'MIRN' instead of 'MIR' but still represents the same gene.",
+"reason": "MIRN95 is an alternate abbreviation of microRNA 95, as it uses 'MIRN' instead of 'MIR' but still represents the same microRNA.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18482,7 +18484,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18565,7 +18567,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18651,7 +18653,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18737,7 +18739,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18778,7 +18780,7 @@
       <c r="L219" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'mir-491' is a lowercase version of the primary gene symbol 'MIR491' and represents the same microRNA gene.",
+"reason": "The alias symbol 'mir-491' is an alternate abbreviation of the official gene name 'microRNA 491' as it uses lowercase letters and a hyphen instead of uppercase letters.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -18823,7 +18825,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18906,7 +18908,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -18947,7 +18949,7 @@
       <c r="L221" t="inlineStr">
         <is>
           <t>{
-"reason": "RanBP2L2 is not an alternate abbreviation because it represents a different description of the gene (RANBP2 like) rather than an abbreviation of the official gene name.",
+"reason": "RanBP2L2 is not an alternate abbreviation of the official gene name because it represents a different description or previous name of the gene, not just a variant abbreviation of 'RANBP2 like and GRIP domain containing 6'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -18992,7 +18994,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19075,7 +19077,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19161,7 +19163,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19202,7 +19204,7 @@
       <c r="L224" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol SNORA25A is not an alternate abbreviation because it includes an additional 'A' character that is not present in the official gene name or primary symbol.",
+"reason": "The alias symbol SNORA25A is not an alternate abbreviation because it contains an additional 'A' character that is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -19247,7 +19249,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19333,7 +19335,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19416,7 +19418,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19502,7 +19504,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19585,7 +19587,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19626,7 +19628,7 @@
       <c r="L229" t="inlineStr">
         <is>
           <t>{
-"reason": "MIRN411 is an alternate abbreviation of microRNA 411, as it uses 'MIRN' instead of 'MIR' to represent 'microRNA' while retaining the same number.",
+"reason": "MIRN411 is an alternate abbreviation of microRNA 411, as it uses 'MIRN' instead of 'MIR' but still represents the same gene.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -19671,7 +19673,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19706,7 +19708,7 @@
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L230" t="inlineStr">
@@ -19754,7 +19756,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19789,7 +19791,7 @@
       </c>
       <c r="K231" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L231" t="inlineStr">
@@ -19837,7 +19839,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19920,7 +19922,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -19961,7 +19963,7 @@
       <c r="L233" t="inlineStr">
         <is>
           <t>{
-"reason": "ELA1 is an alternate abbreviation of CELA1 as it represents the same gene (chymotrypsin like elastase 1) using different letters.",
+"reason": "ELA1 is an alternate abbreviation of the official gene name 'chymotrypsin like elastase 1' as it uses the first letter of 'elastase' and the number '1' from the full name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20006,7 +20008,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20089,7 +20091,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20130,7 +20132,7 @@
       <c r="L235" t="inlineStr">
         <is>
           <t>{
-"reason": "CT45-4 is not an alternate abbreviation because it represents a different member of the CT45 family (CT45-4) compared to the official gene (CT45A5).",
+"reason": "CT45-4 is not an alternate abbreviation because it represents a different member of the CT45 family (CT45-4) rather than specifically referring to CT45A5.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -20175,7 +20177,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20210,7 +20212,7 @@
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L236" t="inlineStr">
@@ -20258,7 +20260,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20341,7 +20343,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20424,7 +20426,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20510,7 +20512,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20596,7 +20598,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20682,7 +20684,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20723,7 +20725,7 @@
       <c r="L242" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'tRNA-Ala-AGC-13-1' is an expanded version of the official gene name 'tRNA-Ala (anticodon AGC) 13-1', using the same components in a slightly different format.",
+"reason": "The alias symbol 'tRNA-Ala-AGC-13-1' is an expanded version of the official gene name 'tRNA-Ala (anticodon AGC) 13-1' with the same meaning and information.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20768,7 +20770,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20809,7 +20811,7 @@
       <c r="L243" t="inlineStr">
         <is>
           <t>{
-"reason": "TRNAD18 is not an alternate abbreviation of the official gene name 'tRNA-Asp (anticodon GTC) 2-1' as it contains characters (18) not present in the official name and does not represent the same gene description.",
+"reason": "TRNAD18 is not an alternate abbreviation of the official gene name 'tRNA-Asp (anticodon GTC) 2-1' as it contains characters (18) not present in the official name and represents a different naming convention.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -20854,7 +20856,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -20895,7 +20897,7 @@
       <c r="L244" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'nmt-tRNA-Gln-TTG-7-1' is an expanded version of the primary gene symbol 'NMTRQ-TTG7-1', representing the same gene with a more descriptive abbreviation that matches the official gene name.",
+"reason": "The alias symbol 'nmt-tRNA-Gln-TTG-7-1' is an expanded version of the primary gene symbol 'NMTRQ-TTG7-1', representing the same gene with a more descriptive format that matches the official gene name.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -20940,7 +20942,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21026,7 +21028,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21112,7 +21114,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21140,22 +21142,19 @@
         </is>
       </c>
       <c r="I247" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J247" t="n">
-        <v>0.5714285714285714</v>
+        <v>0</v>
       </c>
       <c r="K247" t="inlineStr">
         <is>
-          <t>passed_filters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>{
-"reason": "The alias symbol HSA-MIR-548H-1 is an alternate abbreviation of the official gene name 'microRNA 548h-1' with added hyphens and 'HSA' prefix.",
-"alternate_abbreviation": "TRUE"
-}</t>
+          <t>{"alternate_abbreviation": "FALSE"}</t>
         </is>
       </c>
     </row>
@@ -21198,7 +21197,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21239,7 +21238,7 @@
       <c r="L248" t="inlineStr">
         <is>
           <t>{
-"reason": "PAR1 is not derived from the official gene name 'coagulation factor II thrombin receptor' or the primary symbol F2R, but rather stands for 'protease-activated receptor 1', which is a different description of the gene's function.",
+"reason": "PAR1 is not an alternate abbreviation of the official gene name 'coagulation factor II thrombin receptor' as it represents a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21284,7 +21283,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21319,7 +21318,7 @@
       </c>
       <c r="K249" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L249" t="inlineStr">
@@ -21367,7 +21366,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21408,7 +21407,7 @@
       <c r="L250" t="inlineStr">
         <is>
           <t>{
-"reason": "FAT is not an alternate abbreviation because it is a shortened version of the primary gene symbol FAT1, likely representing a family name rather than a specific gene.",
+"reason": "FAT is not an alternate abbreviation because it is a shortened version of the primary gene symbol FAT1, which likely represents a gene family name rather than an abbreviation variant of the specific gene FAT1.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21453,7 +21452,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21536,7 +21535,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21619,7 +21618,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21660,7 +21659,7 @@
       <c r="L253" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol FGF-17 is an alternate abbreviation of the primary gene symbol FGF17, with the only difference being the addition of a hyphen.",
+"reason": "The alias symbol FGF-17 is an alternate abbreviation of the official gene name because it represents the same gene with a hyphen added between FGF and 17.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -21705,7 +21704,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21746,7 +21745,7 @@
       <c r="L254" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL26_10_1113 contains additional characters (_10_1113) not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L26 pseudogene 30'.",
+"reason": "The alias symbol RPL26_10_1113 contains additional characters and numbers not present in the official gene name, indicating it is not an alternate abbreviation of 'ribosomal protein L26 pseudogene 30'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21791,7 +21790,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21874,7 +21873,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -21915,7 +21914,7 @@
       <c r="L256" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol RPL39_3_134 is not an alternate abbreviation because it contains additional characters (_3_134) that are not present in the official gene name or primary symbol.",
+"reason": "The alias symbol RPL39_3_134 is not an alternate abbreviation of the official gene name because it contains additional characters (_3_134) that are not present in the official name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -21960,7 +21959,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22043,7 +22042,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22084,7 +22083,7 @@
       <c r="L258" t="inlineStr">
         <is>
           <t>{
-"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because it represents a different member of the FKBP family (FKBP9 vs FKBP1B).",
+"reason": "FKBP9 is not an alternate abbreviation of FKBP prolyl isomerase 1B because the number 9 in the alias symbol does not match the 1B in the official gene name, indicating it likely refers to a different member of the FKBP gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -22129,7 +22128,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22215,7 +22214,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22298,7 +22297,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22339,7 +22338,7 @@
       <c r="L261" t="inlineStr">
         <is>
           <t>{
-"reason": "FRgamma is an alternate abbreviation as it represents 'folate receptor gamma' using different letters than the primary symbol FOLR3.",
+"reason": "FRgamma is an alternate abbreviation as it represents 'folate receptor gamma' using different letters (FR) for 'folate receptor' and the Greek letter gamma for 'gamma'.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -22384,7 +22383,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22419,7 +22418,7 @@
       </c>
       <c r="K262" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L262" t="inlineStr">
@@ -22467,7 +22466,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22508,7 +22507,7 @@
       <c r="L263" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'mir-3151' is a lowercase version of the primary gene symbol 'MIR3151', representing the same microRNA.",
+"reason": "The alias symbol 'mir-3151' is an alternate abbreviation of the official gene name 'microRNA 3151' as it represents the same gene with a slight variation in capitalization and hyphenation.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -22553,7 +22552,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22636,7 +22635,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22671,7 +22670,7 @@
       </c>
       <c r="K265" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L265" t="inlineStr">
@@ -22719,7 +22718,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22754,7 +22753,7 @@
       </c>
       <c r="K266" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L266" t="inlineStr">
@@ -22802,7 +22801,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22888,7 +22887,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -22971,7 +22970,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23054,7 +23053,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23137,7 +23136,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23172,7 +23171,7 @@
       </c>
       <c r="K271" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L271" t="inlineStr">
@@ -23220,7 +23219,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23255,7 +23254,7 @@
       </c>
       <c r="K272" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L272" t="inlineStr">
@@ -23303,7 +23302,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23386,7 +23385,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23469,7 +23468,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23552,7 +23551,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23593,7 +23592,7 @@
       <c r="L276" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol DDX3YP1 is not an alternate abbreviation because it contains a 'Y' character that is not present in the official gene name or primary symbol.",
+"reason": "The alias symbol DDX3YP1 is not an alternate abbreviation because it contains a 'Y' that is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -23638,7 +23637,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23721,7 +23720,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23762,7 +23761,7 @@
       <c r="L278" t="inlineStr">
         <is>
           <t>{
-"reason": "ALOX12P is not an alternate abbreviation because it lacks the number '1' present in the primary gene symbol ALOX12P1, indicating it may refer to a different gene or gene family.",
+"reason": "ALOX12P is not an alternate abbreviation because it lacks the number '1' present in the primary gene symbol ALOX12P1, which indicates a different gene in the same family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -23807,7 +23806,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23848,7 +23847,7 @@
       <c r="L279" t="inlineStr">
         <is>
           <t>{
-"reason": "RN5S434 is an alternate abbreviation of RNA5SP434 as it represents the same gene with a shortened form of the primary symbol.",
+"reason": "RN5S434 is an alternate abbreviation of RNA5SP434, as it represents the same gene with a shortened form of the primary symbol.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -23893,7 +23892,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -23928,7 +23927,7 @@
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L280" t="inlineStr">
@@ -23976,7 +23975,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24017,7 +24016,7 @@
       <c r="L281" t="inlineStr">
         <is>
           <t>{
-"reason": "HPPO is not derived from the official gene name 'alkaline phosphatase, biomineralization associated' or the primary symbol ALPL, and likely represents a different description of the gene's function.",
+"reason": "HPPO is not an alternate abbreviation of 'alkaline phosphatase, biomineralization associated' as it appears to represent a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -24062,7 +24061,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24145,7 +24144,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24228,7 +24227,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24311,7 +24310,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24394,7 +24393,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24435,7 +24434,7 @@
       <c r="L286" t="inlineStr">
         <is>
           <t>{
-"reason": "GSHPx-3 is an alternate abbreviation of glutathione peroxidase 3, as it represents the same enzyme with a different abbreviation style.",
+"reason": "GSHPx-3 is an alternate abbreviation of glutathione peroxidase 3, as it includes additional characters (SH) and a hyphen that represent the same enzyme but with a slightly different notation.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -24480,7 +24479,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24563,7 +24562,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24646,7 +24645,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24687,7 +24686,7 @@
       <c r="L289" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol H4C3 is not an alternate abbreviation because it represents a different gene (H4 clustered histone 3) than the official gene name (H4 clustered histone 2).",
+"reason": "The alias symbol H4C3 is not an alternate abbreviation of the official gene name 'H4 clustered histone 2' because it represents a different gene within the same family (H4C3 vs H4C2).",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -24732,7 +24731,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24815,7 +24814,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24898,7 +24897,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -24939,7 +24938,7 @@
       <c r="L292" t="inlineStr">
         <is>
           <t>{
-"reason": "SCHAD is not derived from the letters in the official gene name 'hydroxysteroid 17-beta dehydrogenase 10' or the primary symbol 'HSD17B10', suggesting it represents a different description of the gene.",
+"reason": "SCHAD is not derived from the letters in the official gene name 'hydroxysteroid 17-beta dehydrogenase 10' or the primary symbol 'HSD17B10', suggesting it represents a different description or previous name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -24984,7 +24983,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25067,7 +25066,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25150,7 +25149,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25233,7 +25232,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25274,7 +25273,7 @@
       <c r="L296" t="inlineStr">
         <is>
           <t>{
-"reason": "HLAA is an alternate abbreviation of HLA-A as it represents the same gene name without the hyphen.",
+"reason": "HLAA is an alternate abbreviation of HLA-A as it represents the same gene name but without the hyphen.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -25319,7 +25318,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25360,7 +25359,7 @@
       <c r="L297" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol 'onco-lncRNA-32' is not an alternate abbreviation of the official gene name as it includes additional descriptive elements ('onco' and '32') not present in the official name.",
+"reason": "The alias symbol 'onco-lncRNA-32' is not an alternate abbreviation of the official gene name as it includes additional descriptive elements ('onco' and '32') not present in the official name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25405,7 +25404,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25446,7 +25445,7 @@
       <c r="L298" t="inlineStr">
         <is>
           <t>{
-"reason": "A1B is a shortened version of the primary gene symbol A1BG and represents the same gene without introducing new characters.",
+"reason": "A1B is a shortened version of the primary gene symbol A1BG, representing the same gene without altering the meaning.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -25491,7 +25490,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25577,7 +25576,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25618,7 +25617,7 @@
       <c r="L300" t="inlineStr">
         <is>
           <t>{
-"reason": "GAB is not derived from the letters in the official gene name 'alpha-1-B glycoprotein' or the primary symbol 'A1BG'.",
+"reason": "GAB is not an alternate abbreviation of 'alpha-1-B glycoprotein' as it does not represent the same gene name using different letters.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -25663,7 +25662,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25698,7 +25697,7 @@
       </c>
       <c r="K301" t="inlineStr">
         <is>
-          <t>extra_characters</t>
+          <t>hsa_prefix</t>
         </is>
       </c>
       <c r="L301" t="inlineStr">
@@ -25746,7 +25745,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25829,7 +25828,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25912,7 +25911,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -25995,7 +25994,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26078,7 +26077,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26119,7 +26118,7 @@
       <c r="L306" t="inlineStr">
         <is>
           <t>{
-"reason": "HTN5 is not an alternate abbreviation of HTN3 or histatin 3 because the number 5 indicates a different gene in the histatin family.",
+"reason": "HTN5 is not an alternate abbreviation of histatin 3 because the number 5 in the alias symbol represents a different gene in the histatin family than HTN3.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -26164,7 +26163,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26247,7 +26246,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26330,7 +26329,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26413,7 +26412,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26496,7 +26495,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26579,7 +26578,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26665,7 +26664,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26748,7 +26747,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26831,7 +26830,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -26872,7 +26871,7 @@
       <c r="L315" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' with a hyphen added between IL and 12A.",
+"reason": "The alias symbol IL-12A is an alternate abbreviation of the official gene name 'interleukin 12A' as it represents the same gene with a hyphen added between IL and 12A.",
 "alternate_abbreviation": "TRUE"
 }</t>
         </is>
@@ -26917,7 +26916,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27000,7 +26999,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27041,7 +27040,7 @@
       <c r="L317" t="inlineStr">
         <is>
           <t>{
-"reason": "The alias symbol ITGB1BP is not an alternate abbreviation because it lacks the number '2' present in the primary gene symbol ITGB1BP2, which indicates it may represent a different gene or gene family.",
+"reason": "ITGB1BP is not an alternate abbreviation because it lacks the '2' at the end, which is present in both the primary gene symbol and the official gene name, indicating it may represent a different or broader gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -27086,7 +27085,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27169,7 +27168,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27210,7 +27209,7 @@
       <c r="L319" t="inlineStr">
         <is>
           <t>{
-"reason": "LIT1 is not derived from the letters in the official gene name or primary symbol, and appears to represent a different description of the gene.",
+"reason": "LIT1 is not derived from the letters in the official gene name or primary symbol, and appears to be a distinct alias rather than an abbreviation variant.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -27255,7 +27254,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27296,8 +27295,8 @@
       <c r="L320" t="inlineStr">
         <is>
           <t>{
-"reason": "EKLF is an alternate abbreviation for 'Erythroid Kruppel-like Factor', which is a previous name for KLF1, while KLF1 is the current primary gene symbol.",
-"alternate_abbreviation": "TRUE"
+"reason": "EKLF/KLF1 is not an alternate abbreviation because EKLF represents a previous name (Erythroid Kruppel-like Factor) of the gene, while KLF1 is the current primary gene symbol.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -27341,7 +27340,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27382,8 +27381,8 @@
       <c r="L321" t="inlineStr">
         <is>
           <t>{
-"reason": "IPOA7 is an alternate abbreviation for 'importin alpha 7', which is a previous name for karyopherin subunit alpha 6, representing the same gene with different terminology.",
-"alternate_abbreviation": "TRUE"
+"reason": "IPOA7 is an alternate abbreviation for 'importin alpha 7', which was a previous name for this gene and not the current official gene name 'karyopherin subunit alpha 6'.",
+"alternate_abbreviation": "FALSE"
 }</t>
         </is>
       </c>
@@ -27427,7 +27426,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27510,7 +27509,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27593,7 +27592,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27676,7 +27675,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27759,7 +27758,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27842,7 +27841,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -27883,7 +27882,7 @@
       <c r="L327" t="inlineStr">
         <is>
           <t>{
-"reason": "SAMS1 is not an alternate abbreviation of 'methionine adenosyltransferase 1A' as it represents a different description of the gene (S-adenosylmethionine synthetase 1) rather than a variant abbreviation of the official name.",
+"reason": "SAMS1 is not an alternate abbreviation of 'methionine adenosyltransferase 1A' as it represents a different description (S-adenosylmethionine synthetase 1) rather than an abbreviation of the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -27928,7 +27927,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28011,7 +28010,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28094,7 +28093,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28177,7 +28176,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28260,7 +28259,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28343,7 +28342,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28384,7 +28383,7 @@
       <c r="L333" t="inlineStr">
         <is>
           <t>{
-"reason": "MOCS1P2 is not an alternate abbreviation of MOCS1P1 or the official gene name because it represents a different pseudogene (P2 instead of P1) in the same gene family.",
+"reason": "MOCS1P2 is not an alternate abbreviation of MOCS1P1 or 'molybdenum cofactor synthesis 1 pseudogene 1' because it represents a different pseudogene (P2 instead of P1) in the same gene family.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -28429,7 +28428,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28512,7 +28511,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28598,7 +28597,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28684,7 +28683,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28767,7 +28766,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28850,7 +28849,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -28891,7 +28890,7 @@
       <c r="L339" t="inlineStr">
         <is>
           <t>{
-"reason": "NFIB3 is not an alternate abbreviation because it includes a number (3) that is not present in the official gene name or primary symbol.",
+"reason": "NFIB3 is not an alternate abbreviation because the '3' in the alias symbol is not present in the official gene name or primary symbol.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -28936,7 +28935,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29019,7 +29018,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29060,7 +29059,7 @@
       <c r="L341" t="inlineStr">
         <is>
           <t>{
-"reason": "GCNF1 is not an alternate abbreviation of the official gene name as it represents a different description (Germ Cell Nuclear Factor) rather than an abbreviation of 'nuclear receptor subfamily 6 group A member 1'.",
+"reason": "GCNF1 is not an alternate abbreviation of the official gene name as it appears to be a different name or previous name for the gene, not derived from the letters in 'nuclear receptor subfamily 6 group A member 1'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29105,7 +29104,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29146,7 +29145,7 @@
       <c r="L342" t="inlineStr">
         <is>
           <t>{
-"reason": "ABP1 is not derived from the letters in the official gene name 'amine oxidase copper containing 1' or the primary symbol AOC1.",
+"reason": "ABP1 is not an alternate abbreviation of 'amine oxidase copper containing 1' as it does not use the same letters or represent the same concept as the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29191,7 +29190,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29232,7 +29231,7 @@
       <c r="L343" t="inlineStr">
         <is>
           <t>{
-"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains characters (L and 211) not present in 'olfactory receptor family 1 subfamily C member 1'.",
+"reason": "ORL211 is not an alternate abbreviation of the official gene name as it contains characters (L and 211) that are not present in the official name 'olfactory receptor family 1 subfamily C member 1'.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -29277,7 +29276,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29360,7 +29359,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29446,7 +29445,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29529,7 +29528,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29612,7 +29611,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29695,7 +29694,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29781,7 +29780,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29864,7 +29863,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -29947,7 +29946,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30030,7 +30029,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30113,7 +30112,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30196,7 +30195,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30279,7 +30278,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30320,7 +30319,7 @@
       <c r="L356" t="inlineStr">
         <is>
           <t>{
-"reason": "Pr1/Pr2 is not an alternate abbreviation of 'proline rich protein HaeIII subfamily 1' as it represents different subfamily members (1 and 2) rather than the specific PRH1 gene.",
+"reason": "Pr1/Pr2 is not an alternate abbreviation of 'proline rich protein HaeIII subfamily 1' as it represents different subfamily members (1 and 2) rather than an abbreviation of the official gene name.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30365,7 +30364,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30448,7 +30447,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30531,7 +30530,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30614,7 +30613,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30655,7 +30654,7 @@
       <c r="L360" t="inlineStr">
         <is>
           <t>{
-"reason": "SPF27 is not derived from the official gene name 'BCAS2 pre-mRNA processing factor' and appears to represent a different description of the gene.",
+"reason": "SPF27 is not derived from the letters in the official gene name 'BCAS2 pre-mRNA processing factor' and appears to represent a different description or previous name for the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30700,7 +30699,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30783,7 +30782,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30866,7 +30865,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -30907,7 +30906,7 @@
       <c r="L363" t="inlineStr">
         <is>
           <t>{
-"reason": "HNRNP-G is not an abbreviation variant of RBMX pseudogene 1 or RBMXP1, as it represents a different description of the gene (heterogeneous nuclear ribonucleoprotein G) rather than an alternate abbreviation of the official name.",
+"reason": "HNRNP-G is not an abbreviation variant of RBMX pseudogene 1 as it represents a different description or previous name of the gene.",
 "alternate_abbreviation": "FALSE"
 }</t>
         </is>
@@ -30952,7 +30951,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -31035,7 +31034,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 
@@ -31076,8 +31075,8 @@
       <c r="L365" t="inlineStr">
         <is>
           <t>{
-"reason": "RECC1 is not an alternate abbreviation of 'replication factor C subunit 1' as it contains a 'C' not present in the official gene name.",
-"alternate_abbreviation": "FALSE"
+"reason": "RECC1 is an alternate abbreviation of 'replication factor C subunit 1' using different letters to represent the same concept.",
+"alternate_abbreviation": "TRUE"
 }</t>
         </is>
       </c>
@@ -31121,7 +31120,7 @@
           <t xml:space="preserve">Role:You are a biomedical gene nomenclature curator trained in HGNC gene identity and alias symbol resolution.
     You will get fired if your accuracy is less than 95%.
     Background: An alternate abbreviation is when an alias symbol represents the same official gene name or the 
-    primary gene symbol but with different letters. If the alias symbol is representing a different description of
+    primary gene symbol but with different letters. If the alias symbol is representing a different description or a previous name of
     the gene then it is not an alternate abbreviation. Be careful with alias symbols that seem to be shortened versions
     of the primary gene symbol, they may be a family name and therefore not an alternate abbreviation. Alias symbols
     have extra characters may be alternate abbreviations unless they have characters that are not present in the official 

</xml_diff>